<commit_message>
Cerrar RF15c completo: agentes, validadores, persistencia, integración y evidencia
</commit_message>
<xml_diff>
--- a/project/requisitos_backlog.xlsx
+++ b/project/requisitos_backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/erp-fraud-data-TFG/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F03E3A58-A324-684D-B93A-B460BCE514DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81347BAE-E32A-9949-8DF0-F10585CA99EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5913,7 +5913,7 @@
       <c r="D270" s="14"/>
       <c r="E270" s="14"/>
     </row>
-    <row r="271" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A271" s="29" t="s">
         <v>361</v>
       </c>
@@ -5923,10 +5923,12 @@
       <c r="C271" s="14">
         <v>2</v>
       </c>
-      <c r="D271" s="14"/>
+      <c r="D271" s="14">
+        <v>2.5</v>
+      </c>
       <c r="E271" s="14"/>
     </row>
-    <row r="272" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A272" s="19"/>
       <c r="B272" s="31" t="s">
         <v>404</v>
@@ -5934,10 +5936,12 @@
       <c r="C272" s="14">
         <v>2</v>
       </c>
-      <c r="D272" s="14"/>
+      <c r="D272" s="14">
+        <v>3</v>
+      </c>
       <c r="E272" s="14"/>
     </row>
-    <row r="273" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A273" s="16"/>
       <c r="B273" s="28" t="s">
         <v>405</v>
@@ -7194,7 +7198,9 @@
       <c r="C415" s="14">
         <v>2</v>
       </c>
-      <c r="D415" s="14"/>
+      <c r="D415" s="14">
+        <v>2</v>
+      </c>
       <c r="E415" s="14"/>
     </row>
     <row r="416" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -7205,7 +7211,9 @@
       <c r="C416" s="14">
         <v>1.5</v>
       </c>
-      <c r="D416" s="14"/>
+      <c r="D416" s="14">
+        <v>1.8</v>
+      </c>
       <c r="E416" s="14"/>
     </row>
     <row r="417" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -7216,7 +7224,9 @@
       <c r="C417" s="14">
         <v>2.5</v>
       </c>
-      <c r="D417" s="14"/>
+      <c r="D417" s="14">
+        <v>2.5</v>
+      </c>
       <c r="E417" s="14"/>
     </row>
     <row r="418" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -7227,7 +7237,9 @@
       <c r="C418" s="8">
         <v>1.5</v>
       </c>
-      <c r="D418" s="14"/>
+      <c r="D418" s="14">
+        <v>1</v>
+      </c>
       <c r="E418" s="14"/>
     </row>
     <row r="419" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -7238,7 +7250,9 @@
       <c r="C419" s="8">
         <v>1.5</v>
       </c>
-      <c r="D419" s="14"/>
+      <c r="D419" s="14">
+        <v>1.5</v>
+      </c>
       <c r="E419" s="14"/>
     </row>
     <row r="420" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -7249,12 +7263,18 @@
       <c r="C420" s="8">
         <v>1</v>
       </c>
+      <c r="D420" s="8">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="421" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="B421" s="8" t="s">
         <v>500</v>
       </c>
       <c r="C421" s="8">
+        <v>1</v>
+      </c>
+      <c r="D421" s="8">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RF14b: cerrar tareas 11-13 y reforzar experimentos/trazabilidad
</commit_message>
<xml_diff>
--- a/project/requisitos_backlog.xlsx
+++ b/project/requisitos_backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/erp-fraud-data-TFG/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F3CF8DA-D5CB-0E49-9E86-F35202163010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A86670-290B-E641-9D85-D77CFCAD4344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="524">
   <si>
     <t>User story</t>
   </si>
@@ -1576,6 +1576,36 @@
   </si>
   <si>
     <t>RF14-18:Actualización pipeline Github</t>
+  </si>
+  <si>
+    <t>PREREQUISITOS:</t>
+  </si>
+  <si>
+    <t>RF14B-P01:Congelar contratos de salida (GraphState/Explanation/Score/Report) y añadir test de compatibilidad retro</t>
+  </si>
+  <si>
+    <t>RF14B-P02:  Centralizar carga de configuración y eliminar defaults duplicados entre CLI y nodos</t>
+  </si>
+  <si>
+    <t>RF14B-P03: Normalizar observabilidad local (logs + métricas + taxonomy de errores) antes de tracing externo</t>
+  </si>
+  <si>
+    <t>RF14B-P04: Definir y ejecutar release gate de regresión pre-LangSmith (subset RF14/RF15/RF15c/RF18)</t>
+  </si>
+  <si>
+    <t>RF14B-P05: Preparar baseline de secretos (`env.example`) y validación de variables obligatorias</t>
+  </si>
+  <si>
+    <t>RF14B-P06: Cerrar checklist pre-LangSmith y adjuntar evidencia en docs/pre_langsmith_checklist.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RF14b-11: Escribir/actualizar tests de integración (pytest) para este requisito</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RF14b-11: Actualizar documentación (README + runbook/docs) describiendo el comportamiento y cómo verificarlo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RF14b-11: Ejecutar verificación de criterios de aceptación y guardar evidencia (artefactos + enlace de traza LangSmith +</t>
   </si>
 </sst>
 </file>
@@ -3153,7 +3183,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:E445"/>
+  <dimension ref="A2:E456"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="71.33203125" style="26" bestFit="1" customWidth="1"/>
@@ -5262,294 +5292,316 @@
       <c r="E212" s="14"/>
     </row>
     <row r="213" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A213" s="16"/>
+      <c r="A213" s="19"/>
       <c r="B213" s="28"/>
       <c r="C213" s="14"/>
       <c r="D213" s="14"/>
       <c r="E213" s="14"/>
     </row>
-    <row r="214" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="29" t="s">
         <v>351</v>
       </c>
-      <c r="B214" s="28" t="s">
-        <v>384</v>
-      </c>
-      <c r="C214" s="14">
-        <v>0.8</v>
-      </c>
+      <c r="B214" s="28"/>
+      <c r="C214" s="14"/>
       <c r="D214" s="14"/>
       <c r="E214" s="14"/>
     </row>
     <row r="215" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="16"/>
       <c r="B215" s="28" t="s">
-        <v>385</v>
-      </c>
-      <c r="C215" s="14">
-        <v>1.2</v>
-      </c>
+        <v>514</v>
+      </c>
+      <c r="C215" s="14"/>
       <c r="D215" s="14"/>
       <c r="E215" s="14"/>
     </row>
     <row r="216" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="16"/>
       <c r="B216" s="28" t="s">
-        <v>386</v>
+        <v>515</v>
       </c>
       <c r="C216" s="14">
-        <v>1</v>
-      </c>
-      <c r="D216" s="14"/>
+        <v>1.2</v>
+      </c>
+      <c r="D216" s="14">
+        <v>1.8</v>
+      </c>
       <c r="E216" s="14"/>
     </row>
     <row r="217" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="16"/>
       <c r="B217" s="28" t="s">
-        <v>387</v>
+        <v>516</v>
       </c>
       <c r="C217" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="D217" s="14"/>
+        <v>1.2</v>
+      </c>
+      <c r="D217" s="14">
+        <v>2</v>
+      </c>
       <c r="E217" s="14"/>
     </row>
     <row r="218" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218" s="16"/>
       <c r="B218" s="28" t="s">
-        <v>388</v>
+        <v>517</v>
       </c>
       <c r="C218" s="14">
-        <v>2.5</v>
-      </c>
-      <c r="D218" s="14"/>
+        <v>1</v>
+      </c>
+      <c r="D218" s="14">
+        <v>1.8</v>
+      </c>
       <c r="E218" s="14"/>
     </row>
     <row r="219" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="16"/>
       <c r="B219" s="28" t="s">
-        <v>389</v>
+        <v>518</v>
       </c>
       <c r="C219" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D219" s="14"/>
+        <v>1</v>
+      </c>
+      <c r="D219" s="14">
+        <v>1.5</v>
+      </c>
       <c r="E219" s="14"/>
     </row>
     <row r="220" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220" s="16"/>
       <c r="B220" s="28" t="s">
-        <v>390</v>
+        <v>519</v>
       </c>
       <c r="C220" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D220" s="14"/>
+        <v>0.8</v>
+      </c>
+      <c r="D220" s="14">
+        <v>1.5</v>
+      </c>
       <c r="E220" s="14"/>
     </row>
     <row r="221" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A221" s="19"/>
-      <c r="B221" s="31" t="s">
-        <v>391</v>
+      <c r="A221" s="16"/>
+      <c r="B221" s="28" t="s">
+        <v>520</v>
       </c>
       <c r="C221" s="14">
-        <v>2</v>
-      </c>
-      <c r="D221" s="14"/>
+        <v>0.5</v>
+      </c>
+      <c r="D221" s="14">
+        <v>0.5</v>
+      </c>
       <c r="E221" s="14"/>
     </row>
-    <row r="222" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A222" s="16"/>
+    <row r="222" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A222" s="8"/>
       <c r="B222" s="28" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="C222" s="14">
-        <v>1.2</v>
-      </c>
-      <c r="D222" s="14"/>
+        <v>0.8</v>
+      </c>
+      <c r="D222" s="14">
+        <v>1</v>
+      </c>
       <c r="E222" s="14"/>
     </row>
     <row r="223" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223" s="16"/>
       <c r="B223" s="28" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="C223" s="14">
-        <v>1</v>
-      </c>
-      <c r="D223" s="14"/>
+        <v>1.2</v>
+      </c>
+      <c r="D223" s="14">
+        <v>2</v>
+      </c>
       <c r="E223" s="14"/>
     </row>
     <row r="224" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A224" s="16"/>
-      <c r="B224" s="28"/>
-      <c r="C224" s="14"/>
-      <c r="D224" s="14"/>
+      <c r="B224" s="28" t="s">
+        <v>386</v>
+      </c>
+      <c r="C224" s="14">
+        <v>1</v>
+      </c>
+      <c r="D224" s="14">
+        <v>2.5</v>
+      </c>
       <c r="E224" s="14"/>
     </row>
-    <row r="225" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A225" s="29" t="s">
-        <v>354</v>
-      </c>
+    <row r="225" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A225" s="16"/>
       <c r="B225" s="28" t="s">
-        <v>448</v>
+        <v>387</v>
       </c>
       <c r="C225" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D225" s="14"/>
+        <v>0.8</v>
+      </c>
+      <c r="D225" s="14">
+        <v>1</v>
+      </c>
       <c r="E225" s="14"/>
     </row>
-    <row r="226" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226" s="16"/>
       <c r="B226" s="28" t="s">
-        <v>449</v>
+        <v>388</v>
       </c>
       <c r="C226" s="14">
-        <v>0.6</v>
-      </c>
-      <c r="D226" s="14"/>
+        <v>2.5</v>
+      </c>
+      <c r="D226" s="14">
+        <v>0</v>
+      </c>
       <c r="E226" s="14"/>
     </row>
-    <row r="227" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A227" s="16"/>
       <c r="B227" s="28" t="s">
-        <v>450</v>
+        <v>389</v>
       </c>
       <c r="C227" s="14">
-        <v>0.6</v>
-      </c>
-      <c r="D227" s="14"/>
+        <v>1.5</v>
+      </c>
+      <c r="D227" s="14">
+        <v>0</v>
+      </c>
       <c r="E227" s="14"/>
     </row>
-    <row r="228" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A228" s="16"/>
       <c r="B228" s="28" t="s">
-        <v>451</v>
+        <v>390</v>
       </c>
       <c r="C228" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="D228" s="14"/>
+        <v>1.5</v>
+      </c>
+      <c r="D228" s="14">
+        <v>1.8</v>
+      </c>
       <c r="E228" s="14"/>
     </row>
     <row r="229" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A229" s="16"/>
-      <c r="B229" s="28" t="s">
-        <v>452</v>
+      <c r="A229" s="19"/>
+      <c r="B229" s="31" t="s">
+        <v>391</v>
       </c>
       <c r="C229" s="14">
-        <v>1.2</v>
-      </c>
-      <c r="D229" s="14"/>
+        <v>2</v>
+      </c>
+      <c r="D229" s="14">
+        <v>2.5</v>
+      </c>
       <c r="E229" s="14"/>
     </row>
     <row r="230" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A230" s="16"/>
       <c r="B230" s="28" t="s">
-        <v>453</v>
+        <v>392</v>
       </c>
       <c r="C230" s="14">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="D230" s="14"/>
       <c r="E230" s="14"/>
     </row>
     <row r="231" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A231" s="19"/>
+      <c r="A231" s="16"/>
       <c r="B231" s="28" t="s">
-        <v>454</v>
+        <v>393</v>
       </c>
       <c r="C231" s="14">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="D231" s="14"/>
       <c r="E231" s="14"/>
     </row>
-    <row r="232" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A232" s="16"/>
-      <c r="B232" s="31" t="s">
-        <v>455</v>
+      <c r="B232" s="8" t="s">
+        <v>521</v>
       </c>
       <c r="C232" s="14">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="D232" s="14"/>
       <c r="E232" s="14"/>
     </row>
-    <row r="233" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A233" s="16"/>
-      <c r="B233" s="28" t="s">
-        <v>456</v>
+      <c r="B233" s="8" t="s">
+        <v>522</v>
       </c>
       <c r="C233" s="14">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="D233" s="14"/>
       <c r="E233" s="14"/>
     </row>
-    <row r="234" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A234" s="16"/>
-      <c r="B234" s="28" t="s">
-        <v>457</v>
+      <c r="B234" s="8" t="s">
+        <v>523</v>
       </c>
       <c r="C234" s="14">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="D234" s="14"/>
       <c r="E234" s="14"/>
     </row>
     <row r="235" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235" s="16"/>
-      <c r="B235" s="28" t="s">
-        <v>458</v>
-      </c>
-      <c r="C235" s="14">
-        <v>1.5</v>
-      </c>
+      <c r="B235" s="28"/>
+      <c r="C235" s="14"/>
       <c r="D235" s="14"/>
       <c r="E235" s="14"/>
     </row>
-    <row r="236" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A236" s="16"/>
+    <row r="236" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A236" s="29" t="s">
+        <v>354</v>
+      </c>
       <c r="B236" s="28" t="s">
-        <v>459</v>
+        <v>448</v>
       </c>
       <c r="C236" s="14">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D236" s="14"/>
       <c r="E236" s="14"/>
     </row>
-    <row r="237" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A237" s="16"/>
       <c r="B237" s="28" t="s">
-        <v>460</v>
+        <v>449</v>
       </c>
       <c r="C237" s="14">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="D237" s="14"/>
       <c r="E237" s="14"/>
     </row>
-    <row r="238" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A238" s="16"/>
       <c r="B238" s="28" t="s">
-        <v>461</v>
+        <v>450</v>
       </c>
       <c r="C238" s="14">
-        <v>1.2</v>
+        <v>0.6</v>
       </c>
       <c r="D238" s="14"/>
       <c r="E238" s="14"/>
     </row>
-    <row r="239" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A239" s="16"/>
       <c r="B239" s="28" t="s">
-        <v>462</v>
+        <v>451</v>
       </c>
       <c r="C239" s="14">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="D239" s="14"/>
       <c r="E239" s="14"/>
@@ -5557,7 +5609,7 @@
     <row r="240" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240" s="16"/>
       <c r="B240" s="28" t="s">
-        <v>463</v>
+        <v>452</v>
       </c>
       <c r="C240" s="14">
         <v>1.2</v>
@@ -5568,188 +5620,168 @@
     <row r="241" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A241" s="16"/>
       <c r="B241" s="28" t="s">
-        <v>464</v>
+        <v>453</v>
       </c>
       <c r="C241" s="14">
-        <v>2.2000000000000002</v>
+        <v>2</v>
       </c>
       <c r="D241" s="14"/>
       <c r="E241" s="14"/>
     </row>
     <row r="242" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A242" s="16"/>
+      <c r="A242" s="19"/>
       <c r="B242" s="28" t="s">
-        <v>483</v>
+        <v>454</v>
       </c>
       <c r="C242" s="14">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="D242" s="14"/>
       <c r="E242" s="14"/>
     </row>
-    <row r="243" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A243" s="16"/>
-      <c r="B243" s="28" t="s">
-        <v>484</v>
+      <c r="B243" s="31" t="s">
+        <v>455</v>
       </c>
       <c r="C243" s="14">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="D243" s="14"/>
       <c r="E243" s="14"/>
     </row>
-    <row r="244" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A244" s="16" t="s">
-        <v>447</v>
-      </c>
+    <row r="244" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A244" s="16"/>
       <c r="B244" s="28" t="s">
-        <v>485</v>
+        <v>456</v>
       </c>
       <c r="C244" s="14">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="D244" s="14"/>
       <c r="E244" s="14"/>
     </row>
     <row r="245" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245" s="16"/>
-      <c r="B245" s="28"/>
-      <c r="C245" s="14"/>
+      <c r="B245" s="28" t="s">
+        <v>457</v>
+      </c>
+      <c r="C245" s="14">
+        <v>1.8</v>
+      </c>
       <c r="D245" s="14"/>
       <c r="E245" s="14"/>
     </row>
-    <row r="246" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A246" s="32" t="s">
-        <v>355</v>
-      </c>
-      <c r="B246" s="31" t="s">
-        <v>427</v>
+    <row r="246" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A246" s="16"/>
+      <c r="B246" s="28" t="s">
+        <v>458</v>
       </c>
       <c r="C246" s="14">
         <v>1.5</v>
       </c>
-      <c r="D246" s="14">
-        <v>1</v>
-      </c>
+      <c r="D246" s="14"/>
       <c r="E246" s="14"/>
     </row>
-    <row r="247" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247" s="16"/>
       <c r="B247" s="28" t="s">
-        <v>428</v>
+        <v>459</v>
       </c>
       <c r="C247" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D247" s="14">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D247" s="14"/>
       <c r="E247" s="14"/>
     </row>
     <row r="248" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A248" s="16"/>
       <c r="B248" s="28" t="s">
-        <v>429</v>
+        <v>460</v>
       </c>
       <c r="C248" s="14">
-        <v>2</v>
-      </c>
-      <c r="D248" s="14">
-        <v>2</v>
-      </c>
+        <v>0.8</v>
+      </c>
+      <c r="D248" s="14"/>
       <c r="E248" s="14"/>
     </row>
     <row r="249" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249" s="16"/>
       <c r="B249" s="28" t="s">
-        <v>430</v>
+        <v>461</v>
       </c>
       <c r="C249" s="14">
-        <v>2</v>
-      </c>
-      <c r="D249" s="14">
-        <v>2</v>
-      </c>
+        <v>1.2</v>
+      </c>
+      <c r="D249" s="14"/>
       <c r="E249" s="14"/>
     </row>
     <row r="250" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A250" s="16"/>
       <c r="B250" s="28" t="s">
-        <v>431</v>
+        <v>462</v>
       </c>
       <c r="C250" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D250" s="14">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D250" s="14"/>
       <c r="E250" s="14"/>
     </row>
     <row r="251" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251" s="16"/>
       <c r="B251" s="28" t="s">
-        <v>432</v>
+        <v>463</v>
       </c>
       <c r="C251" s="14">
-        <v>1</v>
-      </c>
-      <c r="D251" s="14">
-        <v>0.8</v>
-      </c>
+        <v>1.2</v>
+      </c>
+      <c r="D251" s="14"/>
       <c r="E251" s="14"/>
     </row>
     <row r="252" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252" s="16"/>
       <c r="B252" s="28" t="s">
-        <v>433</v>
+        <v>464</v>
       </c>
       <c r="C252" s="14">
-        <v>2</v>
-      </c>
-      <c r="D252" s="14">
-        <v>2</v>
-      </c>
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D252" s="14"/>
       <c r="E252" s="14"/>
     </row>
     <row r="253" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A253" s="16"/>
       <c r="B253" s="28" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="C253" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D253" s="14">
-        <v>1.5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D253" s="14"/>
       <c r="E253" s="14"/>
     </row>
-    <row r="254" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A254" s="16" t="s">
+    <row r="254" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A254" s="16"/>
+      <c r="B254" s="28" t="s">
+        <v>484</v>
+      </c>
+      <c r="C254" s="14">
+        <v>1</v>
+      </c>
+      <c r="D254" s="14"/>
+      <c r="E254" s="14"/>
+    </row>
+    <row r="255" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A255" s="16" t="s">
         <v>447</v>
       </c>
-      <c r="B254" s="28" t="s">
-        <v>487</v>
-      </c>
-      <c r="C254" s="14">
-        <v>1</v>
-      </c>
-      <c r="D254" s="14">
-        <v>1</v>
-      </c>
-      <c r="E254" s="14"/>
-    </row>
-    <row r="255" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A255" s="16"/>
       <c r="B255" s="28" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="C255" s="14">
         <v>1</v>
       </c>
-      <c r="D255" s="14">
-        <v>1</v>
-      </c>
+      <c r="D255" s="14"/>
       <c r="E255" s="14"/>
     </row>
     <row r="256" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5760,11 +5792,11 @@
       <c r="E256" s="14"/>
     </row>
     <row r="257" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A257" s="29" t="s">
-        <v>358</v>
-      </c>
-      <c r="B257" s="28" t="s">
-        <v>394</v>
+      <c r="A257" s="32" t="s">
+        <v>355</v>
+      </c>
+      <c r="B257" s="31" t="s">
+        <v>427</v>
       </c>
       <c r="C257" s="14">
         <v>1.5</v>
@@ -5774,13 +5806,13 @@
       </c>
       <c r="E257" s="14"/>
     </row>
-    <row r="258" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A258" s="16"/>
       <c r="B258" s="28" t="s">
-        <v>395</v>
+        <v>428</v>
       </c>
       <c r="C258" s="14">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D258" s="14">
         <v>1</v>
@@ -5788,61 +5820,61 @@
       <c r="E258" s="14"/>
     </row>
     <row r="259" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A259" s="19"/>
-      <c r="B259" s="31" t="s">
-        <v>396</v>
+      <c r="A259" s="16"/>
+      <c r="B259" s="28" t="s">
+        <v>429</v>
       </c>
       <c r="C259" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D259" s="14">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="E259" s="14"/>
     </row>
     <row r="260" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="16"/>
       <c r="B260" s="28" t="s">
-        <v>397</v>
+        <v>430</v>
       </c>
       <c r="C260" s="14">
         <v>2</v>
       </c>
       <c r="D260" s="14">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E260" s="14"/>
     </row>
     <row r="261" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="16"/>
       <c r="B261" s="28" t="s">
-        <v>398</v>
+        <v>431</v>
       </c>
       <c r="C261" s="14">
         <v>1.5</v>
       </c>
       <c r="D261" s="14">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E261" s="14"/>
     </row>
     <row r="262" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262" s="16"/>
       <c r="B262" s="28" t="s">
-        <v>399</v>
+        <v>432</v>
       </c>
       <c r="C262" s="14">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="D262" s="14">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="E262" s="14"/>
     </row>
     <row r="263" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="16"/>
       <c r="B263" s="28" t="s">
-        <v>400</v>
+        <v>433</v>
       </c>
       <c r="C263" s="14">
         <v>2</v>
@@ -5855,33 +5887,35 @@
     <row r="264" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="16"/>
       <c r="B264" s="28" t="s">
-        <v>401</v>
+        <v>486</v>
       </c>
       <c r="C264" s="14">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D264" s="14">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E264" s="14"/>
     </row>
     <row r="265" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A265" s="16"/>
+      <c r="A265" s="16" t="s">
+        <v>447</v>
+      </c>
       <c r="B265" s="28" t="s">
-        <v>402</v>
+        <v>487</v>
       </c>
       <c r="C265" s="14">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="D265" s="14">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E265" s="14"/>
     </row>
     <row r="266" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266" s="16"/>
       <c r="B266" s="28" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="C266" s="14">
         <v>1</v>
@@ -5893,94 +5927,98 @@
     </row>
     <row r="267" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267" s="16"/>
-      <c r="B267" s="28" t="s">
-        <v>481</v>
-      </c>
-      <c r="C267" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="D267" s="14">
-        <v>0.8</v>
-      </c>
+      <c r="B267" s="28"/>
+      <c r="C267" s="14"/>
+      <c r="D267" s="14"/>
       <c r="E267" s="14"/>
     </row>
-    <row r="268" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A268" s="16"/>
+    <row r="268" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A268" s="29" t="s">
+        <v>358</v>
+      </c>
       <c r="B268" s="28" t="s">
-        <v>482</v>
+        <v>394</v>
       </c>
       <c r="C268" s="14">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="D268" s="14">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E268" s="14"/>
     </row>
     <row r="269" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="16"/>
-      <c r="B269" s="28"/>
-      <c r="C269" s="14"/>
-      <c r="D269" s="14"/>
+      <c r="B269" s="28" t="s">
+        <v>395</v>
+      </c>
+      <c r="C269" s="14">
+        <v>1</v>
+      </c>
+      <c r="D269" s="14">
+        <v>1</v>
+      </c>
       <c r="E269" s="14"/>
     </row>
     <row r="270" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A270" s="16" t="s">
-        <v>447</v>
-      </c>
-      <c r="B270" s="28"/>
-      <c r="C270" s="14"/>
-      <c r="D270" s="14"/>
+      <c r="A270" s="19"/>
+      <c r="B270" s="31" t="s">
+        <v>396</v>
+      </c>
+      <c r="C270" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D270" s="14">
+        <v>1.2</v>
+      </c>
       <c r="E270" s="14"/>
     </row>
-    <row r="271" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A271" s="29" t="s">
-        <v>361</v>
-      </c>
+    <row r="271" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A271" s="16"/>
       <c r="B271" s="28" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="C271" s="14">
         <v>2</v>
       </c>
       <c r="D271" s="14">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="E271" s="14"/>
     </row>
-    <row r="272" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A272" s="19"/>
-      <c r="B272" s="31" t="s">
-        <v>404</v>
+    <row r="272" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A272" s="16"/>
+      <c r="B272" s="28" t="s">
+        <v>398</v>
       </c>
       <c r="C272" s="14">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D272" s="14">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="E272" s="14"/>
     </row>
-    <row r="273" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A273" s="16"/>
       <c r="B273" s="28" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="C273" s="14">
         <v>2.5</v>
       </c>
       <c r="D273" s="14">
-        <v>3.8</v>
+        <v>2</v>
       </c>
       <c r="E273" s="14"/>
     </row>
-    <row r="274" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A274" s="16"/>
       <c r="B274" s="28" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
       <c r="C274" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D274" s="14">
         <v>2</v>
@@ -5990,255 +6028,249 @@
     <row r="275" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A275" s="16"/>
       <c r="B275" s="28" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="C275" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D275" s="14">
-        <v>2.2000000000000002</v>
+        <v>1</v>
       </c>
       <c r="E275" s="14"/>
     </row>
-    <row r="276" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A276" s="16"/>
       <c r="B276" s="28" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="C276" s="14">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="D276" s="14">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="E276" s="14"/>
     </row>
     <row r="277" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A277" s="16"/>
       <c r="B277" s="28" t="s">
-        <v>409</v>
+        <v>480</v>
       </c>
       <c r="C277" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D277" s="14">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="E277" s="14"/>
     </row>
-    <row r="278" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A278" s="16"/>
       <c r="B278" s="28" t="s">
-        <v>410</v>
+        <v>481</v>
       </c>
       <c r="C278" s="14">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="D278" s="14">
-        <v>4</v>
+        <v>0.8</v>
       </c>
       <c r="E278" s="14"/>
     </row>
     <row r="279" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A279" s="16"/>
       <c r="B279" s="28" t="s">
-        <v>411</v>
+        <v>482</v>
       </c>
       <c r="C279" s="14">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D279" s="14">
-        <v>2.8</v>
+        <v>0.5</v>
       </c>
       <c r="E279" s="14"/>
     </row>
     <row r="280" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A280" s="16"/>
-      <c r="B280" s="28" t="s">
-        <v>412</v>
-      </c>
-      <c r="C280" s="14">
+      <c r="B280" s="28"/>
+      <c r="C280" s="14"/>
+      <c r="D280" s="14"/>
+      <c r="E280" s="14"/>
+    </row>
+    <row r="281" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A281" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="B281" s="28"/>
+      <c r="C281" s="14"/>
+      <c r="D281" s="14"/>
+      <c r="E281" s="14"/>
+    </row>
+    <row r="282" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A282" s="29" t="s">
+        <v>361</v>
+      </c>
+      <c r="B282" s="28" t="s">
+        <v>403</v>
+      </c>
+      <c r="C282" s="14">
         <v>2</v>
       </c>
-      <c r="D280" s="14">
+      <c r="D282" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="E282" s="14"/>
+    </row>
+    <row r="283" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A283" s="19"/>
+      <c r="B283" s="31" t="s">
+        <v>404</v>
+      </c>
+      <c r="C283" s="14">
         <v>2</v>
       </c>
-      <c r="E280" s="14"/>
-    </row>
-    <row r="281" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A281" s="19"/>
-      <c r="B281" s="31" t="s">
-        <v>413</v>
-      </c>
-      <c r="C281" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D281" s="14">
-        <v>1.2</v>
-      </c>
-      <c r="E281" s="14"/>
-    </row>
-    <row r="282" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A282" s="16"/>
-      <c r="B282" s="28" t="s">
-        <v>414</v>
-      </c>
-      <c r="C282" s="14">
-        <v>1</v>
-      </c>
-      <c r="D282" s="14">
-        <v>1</v>
-      </c>
-      <c r="E282" s="14"/>
-    </row>
-    <row r="283" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A283" s="16"/>
-      <c r="B283" s="28" t="s">
-        <v>415</v>
-      </c>
-      <c r="C283" s="14">
+      <c r="D283" s="14">
         <v>3</v>
       </c>
-      <c r="D283" s="14">
-        <v>2.5</v>
-      </c>
       <c r="E283" s="14"/>
     </row>
-    <row r="284" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A284" s="16"/>
       <c r="B284" s="28" t="s">
-        <v>416</v>
+        <v>405</v>
       </c>
       <c r="C284" s="14">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="D284" s="14">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="E284" s="14"/>
     </row>
-    <row r="285" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A285" s="16"/>
       <c r="B285" s="28" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="C285" s="14">
         <v>1.5</v>
       </c>
       <c r="D285" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E285" s="14"/>
     </row>
     <row r="286" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A286" s="16"/>
       <c r="B286" s="28" t="s">
-        <v>489</v>
-      </c>
-      <c r="C286" s="8">
+        <v>407</v>
+      </c>
+      <c r="C286" s="14">
         <v>2</v>
       </c>
       <c r="D286" s="14">
-        <v>1.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E286" s="14"/>
     </row>
-    <row r="287" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A287" s="16"/>
       <c r="B287" s="28" t="s">
-        <v>490</v>
-      </c>
-      <c r="C287" s="8">
-        <v>1</v>
+        <v>408</v>
+      </c>
+      <c r="C287" s="14">
+        <v>1.5</v>
       </c>
       <c r="D287" s="14">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E287" s="14"/>
     </row>
     <row r="288" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A288" s="16"/>
       <c r="B288" s="28" t="s">
-        <v>491</v>
-      </c>
-      <c r="C288" s="8">
-        <v>1</v>
+        <v>409</v>
+      </c>
+      <c r="C288" s="14">
+        <v>2</v>
       </c>
       <c r="D288" s="14">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="E288" s="14"/>
     </row>
-    <row r="289" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A289" s="16" t="s">
-        <v>447</v>
-      </c>
-      <c r="B289" s="28"/>
-      <c r="C289" s="14"/>
-      <c r="D289" s="14"/>
+    <row r="289" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A289" s="16"/>
+      <c r="B289" s="28" t="s">
+        <v>410</v>
+      </c>
+      <c r="C289" s="14">
+        <v>2</v>
+      </c>
+      <c r="D289" s="14">
+        <v>4</v>
+      </c>
       <c r="E289" s="14"/>
     </row>
-    <row r="290" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A290" s="29" t="s">
-        <v>364</v>
-      </c>
-      <c r="B290" s="18" t="s">
-        <v>418</v>
+    <row r="290" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A290" s="16"/>
+      <c r="B290" s="28" t="s">
+        <v>411</v>
       </c>
       <c r="C290" s="14">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="D290" s="14">
-        <v>0.5</v>
+        <v>2.8</v>
       </c>
       <c r="E290" s="14"/>
     </row>
     <row r="291" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A291" s="16"/>
-      <c r="B291" s="18" t="s">
-        <v>419</v>
+      <c r="B291" s="28" t="s">
+        <v>412</v>
       </c>
       <c r="C291" s="14">
         <v>2</v>
       </c>
       <c r="D291" s="14">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E291" s="14"/>
     </row>
     <row r="292" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A292" s="16"/>
-      <c r="B292" s="18" t="s">
-        <v>420</v>
+      <c r="A292" s="19"/>
+      <c r="B292" s="31" t="s">
+        <v>413</v>
       </c>
       <c r="C292" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D292" s="14">
         <v>1.2</v>
       </c>
-      <c r="D292" s="14">
-        <v>1.5</v>
-      </c>
       <c r="E292" s="14"/>
     </row>
     <row r="293" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A293" s="19"/>
-      <c r="B293" s="14" t="s">
-        <v>421</v>
+      <c r="A293" s="16"/>
+      <c r="B293" s="28" t="s">
+        <v>414</v>
       </c>
       <c r="C293" s="14">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D293" s="14">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="E293" s="14"/>
     </row>
     <row r="294" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A294" s="16"/>
-      <c r="B294" s="18" t="s">
-        <v>422</v>
+      <c r="B294" s="28" t="s">
+        <v>415</v>
       </c>
       <c r="C294" s="14">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D294" s="14">
         <v>2.5</v>
@@ -6247,543 +6279,604 @@
     </row>
     <row r="295" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A295" s="16"/>
-      <c r="B295" s="18" t="s">
-        <v>423</v>
+      <c r="B295" s="28" t="s">
+        <v>416</v>
       </c>
       <c r="C295" s="14">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D295" s="14">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="E295" s="14"/>
     </row>
     <row r="296" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A296" s="16"/>
-      <c r="B296" s="18" t="s">
-        <v>424</v>
+      <c r="B296" s="28" t="s">
+        <v>417</v>
       </c>
       <c r="C296" s="14">
         <v>1.5</v>
       </c>
       <c r="D296" s="14">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E296" s="14"/>
     </row>
     <row r="297" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A297" s="16"/>
-      <c r="B297" s="18" t="s">
-        <v>425</v>
-      </c>
-      <c r="C297" s="14">
-        <v>3</v>
+      <c r="B297" s="28" t="s">
+        <v>489</v>
+      </c>
+      <c r="C297" s="8">
+        <v>2</v>
       </c>
       <c r="D297" s="14">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="E297" s="14"/>
     </row>
     <row r="298" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A298" s="16"/>
-      <c r="B298" s="18" t="s">
-        <v>504</v>
-      </c>
-      <c r="C298" s="14">
-        <v>1.2</v>
+      <c r="B298" s="28" t="s">
+        <v>490</v>
+      </c>
+      <c r="C298" s="8">
+        <v>1</v>
       </c>
       <c r="D298" s="14">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="E298" s="14"/>
     </row>
     <row r="299" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A299" s="16"/>
-      <c r="B299" s="18" t="s">
+      <c r="B299" s="28" t="s">
+        <v>491</v>
+      </c>
+      <c r="C299" s="8">
+        <v>1</v>
+      </c>
+      <c r="D299" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="E299" s="14"/>
+    </row>
+    <row r="300" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A300" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="B300" s="28"/>
+      <c r="C300" s="14"/>
+      <c r="D300" s="14"/>
+      <c r="E300" s="14"/>
+    </row>
+    <row r="301" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A301" s="29" t="s">
+        <v>364</v>
+      </c>
+      <c r="B301" s="18" t="s">
+        <v>418</v>
+      </c>
+      <c r="C301" s="14">
+        <v>0.8</v>
+      </c>
+      <c r="D301" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="E301" s="14"/>
+    </row>
+    <row r="302" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A302" s="16"/>
+      <c r="B302" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="C302" s="14">
+        <v>2</v>
+      </c>
+      <c r="D302" s="14">
+        <v>1.8</v>
+      </c>
+      <c r="E302" s="14"/>
+    </row>
+    <row r="303" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A303" s="16"/>
+      <c r="B303" s="18" t="s">
+        <v>420</v>
+      </c>
+      <c r="C303" s="14">
+        <v>1.2</v>
+      </c>
+      <c r="D303" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E303" s="14"/>
+    </row>
+    <row r="304" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A304" s="19"/>
+      <c r="B304" s="14" t="s">
+        <v>421</v>
+      </c>
+      <c r="C304" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D304" s="14">
+        <v>1.8</v>
+      </c>
+      <c r="E304" s="14"/>
+    </row>
+    <row r="305" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A305" s="16"/>
+      <c r="B305" s="18" t="s">
+        <v>422</v>
+      </c>
+      <c r="C305" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="D305" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="E305" s="14"/>
+    </row>
+    <row r="306" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A306" s="16"/>
+      <c r="B306" s="18" t="s">
+        <v>423</v>
+      </c>
+      <c r="C306" s="14">
+        <v>2</v>
+      </c>
+      <c r="D306" s="14">
+        <v>2</v>
+      </c>
+      <c r="E306" s="14"/>
+    </row>
+    <row r="307" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A307" s="16"/>
+      <c r="B307" s="18" t="s">
+        <v>424</v>
+      </c>
+      <c r="C307" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D307" s="14">
+        <v>1</v>
+      </c>
+      <c r="E307" s="14"/>
+    </row>
+    <row r="308" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A308" s="16"/>
+      <c r="B308" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="C308" s="14">
+        <v>3</v>
+      </c>
+      <c r="D308" s="14">
+        <v>3.5</v>
+      </c>
+      <c r="E308" s="14"/>
+    </row>
+    <row r="309" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A309" s="16"/>
+      <c r="B309" s="18" t="s">
+        <v>504</v>
+      </c>
+      <c r="C309" s="14">
+        <v>1.2</v>
+      </c>
+      <c r="D309" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E309" s="14"/>
+    </row>
+    <row r="310" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A310" s="16"/>
+      <c r="B310" s="18" t="s">
         <v>426</v>
       </c>
-      <c r="C299" s="14">
+      <c r="C310" s="14">
         <v>1.2</v>
       </c>
-      <c r="D299" s="14">
-        <v>1</v>
-      </c>
-      <c r="E299" s="14"/>
-    </row>
-    <row r="300" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A300" s="16"/>
-      <c r="B300" s="18" t="s">
+      <c r="D310" s="14">
+        <v>1</v>
+      </c>
+      <c r="E310" s="14"/>
+    </row>
+    <row r="311" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A311" s="16"/>
+      <c r="B311" s="18" t="s">
         <v>492</v>
       </c>
-      <c r="C300" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D300" s="14">
-        <v>1</v>
-      </c>
-      <c r="E300" s="14"/>
-    </row>
-    <row r="301" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A301" s="16"/>
-      <c r="B301" s="18" t="s">
+      <c r="C311" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D311" s="14">
+        <v>1</v>
+      </c>
+      <c r="E311" s="14"/>
+    </row>
+    <row r="312" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A312" s="16"/>
+      <c r="B312" s="18" t="s">
         <v>493</v>
       </c>
-      <c r="C301" s="14">
-        <v>1</v>
-      </c>
-      <c r="D301" s="8">
+      <c r="C312" s="14">
+        <v>1</v>
+      </c>
+      <c r="D312" s="8">
         <v>0.8</v>
       </c>
     </row>
-    <row r="302" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B302" s="18" t="s">
+    <row r="313" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B313" s="18" t="s">
         <v>494</v>
       </c>
-      <c r="C302" s="14">
-        <v>1</v>
-      </c>
-      <c r="D302" s="8">
+      <c r="C313" s="14">
+        <v>1</v>
+      </c>
+      <c r="D313" s="8">
         <v>0.8</v>
       </c>
     </row>
-    <row r="303" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A303" s="36" t="s">
+    <row r="314" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A314" s="36" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="304" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B304" s="28" t="s">
+    <row r="315" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B315" s="28" t="s">
         <v>240</v>
       </c>
-      <c r="C304" s="8">
+      <c r="C315" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="305" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B305" s="28" t="s">
+    <row r="316" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B316" s="28" t="s">
         <v>241</v>
       </c>
-      <c r="C305" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="306" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B306" s="28" t="s">
+      <c r="C316" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="317" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B317" s="28" t="s">
         <v>242</v>
       </c>
-      <c r="C306" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="307" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B307" s="28" t="s">
+      <c r="C317" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B318" s="28" t="s">
         <v>243</v>
       </c>
-      <c r="C307" s="8">
+      <c r="C318" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="308" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B308" s="28" t="s">
+    <row r="319" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B319" s="28" t="s">
         <v>244</v>
       </c>
-      <c r="C308" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="309" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B309" s="28" t="s">
+      <c r="C319" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B320" s="28" t="s">
         <v>245</v>
       </c>
-      <c r="C309" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="310" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B310" s="28" t="s">
+      <c r="C320" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="321" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B321" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="C310" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="311" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B311" s="28" t="s">
+      <c r="C321" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B322" s="28" t="s">
         <v>247</v>
       </c>
-      <c r="C311" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B312" s="28"/>
-    </row>
-    <row r="313" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A313" s="36" t="s">
+      <c r="C322" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B323" s="28"/>
+    </row>
+    <row r="324" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A324" s="36" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="314" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B314" s="28" t="s">
+    <row r="325" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B325" s="28" t="s">
         <v>248</v>
       </c>
-      <c r="C314" s="8">
+      <c r="C325" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="315" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B315" s="28" t="s">
+    <row r="326" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B326" s="28" t="s">
         <v>249</v>
       </c>
-      <c r="C315" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="316" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B316" s="28" t="s">
+      <c r="C326" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B327" s="28" t="s">
         <v>250</v>
       </c>
-      <c r="C316" s="8">
+      <c r="C327" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="317" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B317" s="28" t="s">
+    <row r="328" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B328" s="28" t="s">
         <v>251</v>
       </c>
-      <c r="C317" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="318" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B318" s="28" t="s">
+      <c r="C328" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="329" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B329" s="28" t="s">
         <v>252</v>
       </c>
-      <c r="C318" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="319" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B319" s="28" t="s">
+      <c r="C329" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="330" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B330" s="28" t="s">
         <v>253</v>
       </c>
-      <c r="C319" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="320" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B320" s="28" t="s">
+      <c r="C330" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="331" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B331" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="C320" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B321" s="28"/>
-    </row>
-    <row r="322" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A322" s="29" t="s">
+      <c r="C331" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="332" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B332" s="28"/>
+    </row>
+    <row r="333" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A333" s="29" t="s">
         <v>367</v>
       </c>
-      <c r="B322" s="28" t="s">
+      <c r="B333" s="28" t="s">
         <v>434</v>
       </c>
-      <c r="C322" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D322" s="14">
+      <c r="C333" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D333" s="14">
         <v>1.2</v>
       </c>
-      <c r="E322" s="14"/>
-    </row>
-    <row r="323" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B323" s="28" t="s">
+      <c r="E333" s="14"/>
+    </row>
+    <row r="334" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B334" s="28" t="s">
         <v>435</v>
       </c>
-      <c r="C323" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D323" s="14">
+      <c r="C334" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D334" s="14">
         <v>2</v>
       </c>
-      <c r="E323" s="14"/>
-    </row>
-    <row r="324" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A324" s="16"/>
-      <c r="B324" s="28" t="s">
+      <c r="E334" s="14"/>
+    </row>
+    <row r="335" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A335" s="16"/>
+      <c r="B335" s="28" t="s">
         <v>436</v>
       </c>
-      <c r="C324" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D324" s="14">
+      <c r="C335" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D335" s="14">
         <v>2</v>
       </c>
-      <c r="E324" s="14"/>
-    </row>
-    <row r="325" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A325" s="16"/>
-      <c r="B325" s="28" t="s">
+      <c r="E335" s="14"/>
+    </row>
+    <row r="336" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A336" s="16"/>
+      <c r="B336" s="28" t="s">
         <v>437</v>
       </c>
-      <c r="C325" s="14">
+      <c r="C336" s="14">
         <v>2</v>
       </c>
-      <c r="D325" s="14">
+      <c r="D336" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="E325" s="14"/>
-    </row>
-    <row r="326" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A326" s="16"/>
-      <c r="B326" s="28" t="s">
+      <c r="E336" s="14"/>
+    </row>
+    <row r="337" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A337" s="16"/>
+      <c r="B337" s="28" t="s">
         <v>438</v>
       </c>
-      <c r="C326" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D326" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="E326" s="14"/>
-    </row>
-    <row r="327" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A327" s="16"/>
-      <c r="B327" s="28" t="s">
+      <c r="C337" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D337" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E337" s="14"/>
+    </row>
+    <row r="338" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A338" s="16"/>
+      <c r="B338" s="28" t="s">
         <v>439</v>
       </c>
-      <c r="C327" s="14">
+      <c r="C338" s="14">
         <v>1.2</v>
       </c>
-      <c r="D327" s="14">
-        <v>1</v>
-      </c>
-      <c r="E327" s="14"/>
-    </row>
-    <row r="328" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A328" s="16"/>
-      <c r="B328" s="28" t="s">
+      <c r="D338" s="14">
+        <v>1</v>
+      </c>
+      <c r="E338" s="14"/>
+    </row>
+    <row r="339" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A339" s="16"/>
+      <c r="B339" s="28" t="s">
         <v>440</v>
       </c>
-      <c r="C328" s="14">
-        <v>1</v>
-      </c>
-      <c r="D328" s="14">
+      <c r="C339" s="14">
+        <v>1</v>
+      </c>
+      <c r="D339" s="14">
         <v>0.8</v>
       </c>
-      <c r="E328" s="14"/>
-    </row>
-    <row r="329" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A329" s="16"/>
-      <c r="B329" s="28" t="s">
+      <c r="E339" s="14"/>
+    </row>
+    <row r="340" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A340" s="16"/>
+      <c r="B340" s="28" t="s">
         <v>441</v>
       </c>
-      <c r="C329" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D329" s="14">
+      <c r="C340" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D340" s="14">
         <v>1.8</v>
       </c>
-      <c r="E329" s="14"/>
-    </row>
-    <row r="330" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A330" s="16"/>
-      <c r="B330" s="28" t="s">
+      <c r="E340" s="14"/>
+    </row>
+    <row r="341" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A341" s="16"/>
+      <c r="B341" s="28" t="s">
         <v>442</v>
       </c>
-      <c r="C330" s="14">
+      <c r="C341" s="14">
         <v>2</v>
       </c>
-      <c r="D330" s="14">
+      <c r="D341" s="14">
         <v>2.5</v>
       </c>
-      <c r="E330" s="14"/>
-    </row>
-    <row r="331" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A331" s="16"/>
-      <c r="B331" s="28" t="s">
+      <c r="E341" s="14"/>
+    </row>
+    <row r="342" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A342" s="16"/>
+      <c r="B342" s="28" t="s">
         <v>443</v>
       </c>
-      <c r="C331" s="14">
-        <v>1</v>
-      </c>
-      <c r="D331" s="14">
-        <v>1</v>
-      </c>
-      <c r="E331" s="14"/>
-    </row>
-    <row r="332" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A332" s="16"/>
-      <c r="B332" s="28" t="s">
+      <c r="C342" s="14">
+        <v>1</v>
+      </c>
+      <c r="D342" s="14">
+        <v>1</v>
+      </c>
+      <c r="E342" s="14"/>
+    </row>
+    <row r="343" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A343" s="16"/>
+      <c r="B343" s="28" t="s">
         <v>495</v>
       </c>
-      <c r="C332" s="8">
-        <v>1.5</v>
-      </c>
-      <c r="D332" s="14">
-        <v>1</v>
-      </c>
-      <c r="E332" s="14"/>
-    </row>
-    <row r="333" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A333" s="16"/>
-      <c r="B333" s="28" t="s">
+      <c r="C343" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="D343" s="14">
+        <v>1</v>
+      </c>
+      <c r="E343" s="14"/>
+    </row>
+    <row r="344" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A344" s="16"/>
+      <c r="B344" s="28" t="s">
         <v>496</v>
       </c>
-      <c r="C333" s="8">
-        <v>1</v>
-      </c>
-      <c r="D333" s="14">
+      <c r="C344" s="8">
+        <v>1</v>
+      </c>
+      <c r="D344" s="14">
         <v>0.8</v>
       </c>
-      <c r="E333" s="14"/>
-    </row>
-    <row r="334" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A334" s="16"/>
-      <c r="B334" s="28" t="s">
+      <c r="E344" s="14"/>
+    </row>
+    <row r="345" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A345" s="16"/>
+      <c r="B345" s="28" t="s">
         <v>497</v>
       </c>
-      <c r="C334" s="8">
-        <v>1</v>
-      </c>
-      <c r="D334" s="8">
+      <c r="C345" s="8">
+        <v>1</v>
+      </c>
+      <c r="D345" s="8">
         <v>0.5</v>
       </c>
-      <c r="E334" s="14"/>
-    </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A335" s="16"/>
-      <c r="B335" s="28"/>
-    </row>
-    <row r="336" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A336" s="36" t="s">
+      <c r="E345" s="14"/>
+    </row>
+    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A346" s="16"/>
+      <c r="B346" s="28"/>
+    </row>
+    <row r="347" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A347" s="36" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="337" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B337" s="28" t="s">
+    <row r="348" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B348" s="28" t="s">
         <v>255</v>
       </c>
-      <c r="C337" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="338" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B338" s="28" t="s">
+      <c r="C348" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="349" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B349" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="C338" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="339" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B339" s="28" t="s">
+      <c r="C349" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="350" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B350" s="28" t="s">
         <v>257</v>
       </c>
-      <c r="C339" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="340" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B340" s="28" t="s">
+      <c r="C350" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="351" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B351" s="28" t="s">
         <v>258</v>
-      </c>
-      <c r="C340" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="341" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B341" s="28" t="s">
-        <v>259</v>
-      </c>
-      <c r="C341" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="342" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B342" s="28" t="s">
-        <v>260</v>
-      </c>
-      <c r="C342" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="343" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B343" s="28" t="s">
-        <v>261</v>
-      </c>
-      <c r="C343" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="344" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B344" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="C344" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="345" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B345" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="C345" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="346" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B346" s="28"/>
-    </row>
-    <row r="347" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A347" s="36" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="348" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B348" s="28" t="s">
-        <v>264</v>
-      </c>
-      <c r="C348" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="349" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B349" s="28" t="s">
-        <v>265</v>
-      </c>
-      <c r="C349" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="350" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B350" s="28" t="s">
-        <v>266</v>
-      </c>
-      <c r="C350" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="351" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B351" s="28" t="s">
-        <v>267</v>
       </c>
       <c r="C351" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="352" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B352" s="28" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="C352" s="8">
         <v>1.5</v>
       </c>
     </row>
-    <row r="353" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B353" s="28" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="C353" s="8">
         <v>1</v>
@@ -6791,183 +6884,183 @@
     </row>
     <row r="354" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B354" s="28" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="C354" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="355" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B355" s="28"/>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B355" s="28" t="s">
+        <v>262</v>
+      </c>
+      <c r="C355" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="356" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A356" s="36" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="357" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B357" s="28" t="s">
-        <v>271</v>
-      </c>
-      <c r="C357" s="8">
-        <v>0.8</v>
-      </c>
+      <c r="B356" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="C356" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B357" s="28"/>
     </row>
     <row r="358" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B358" s="28" t="s">
-        <v>272</v>
-      </c>
-      <c r="C358" s="8">
-        <v>0.8</v>
+      <c r="A358" s="36" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="359" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B359" s="28" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C359" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="360" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B360" s="28" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="C360" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="361" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="361" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B361" s="28" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="C361" s="8">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="362" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B362" s="28" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="C362" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="363" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B363" s="28" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="C363" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="364" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B364" s="28"/>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B364" s="28" t="s">
+        <v>269</v>
+      </c>
+      <c r="C364" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="365" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A365" s="36" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="366" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B366" s="28" t="s">
-        <v>278</v>
-      </c>
-      <c r="C366" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="367" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B367" s="28" t="s">
-        <v>279</v>
-      </c>
-      <c r="C367" s="8">
-        <v>1.5</v>
+      <c r="B365" s="28" t="s">
+        <v>270</v>
+      </c>
+      <c r="C365" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B366" s="28"/>
+    </row>
+    <row r="367" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A367" s="36" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="368" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B368" s="28" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="C368" s="8">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="369" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B369" s="28" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="C369" s="8">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="370" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B370" s="28" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="C370" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="371" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B371" s="28" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="C371" s="8">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="372" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B372" s="28" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="C372" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="373" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B373" s="28"/>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B373" s="28" t="s">
+        <v>276</v>
+      </c>
+      <c r="C373" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="374" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A374" s="36" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="375" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B375" s="28" t="s">
-        <v>285</v>
-      </c>
-      <c r="C375" s="8">
-        <v>1.5</v>
-      </c>
+      <c r="B374" s="28" t="s">
+        <v>277</v>
+      </c>
+      <c r="C374" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B375" s="28"/>
     </row>
     <row r="376" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B376" s="28" t="s">
-        <v>286</v>
-      </c>
-      <c r="C376" s="8">
-        <v>1.5</v>
+      <c r="A376" s="36" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="377" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B377" s="28" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="C377" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="378" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B378" s="28" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C378" s="8">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="379" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="379" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B379" s="28" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="C379" s="8">
         <v>1</v>
@@ -6975,111 +7068,111 @@
     </row>
     <row r="380" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B380" s="28" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C380" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="381" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B381" s="28"/>
-    </row>
-    <row r="382" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A382" s="36" t="s">
-        <v>75</v>
+    <row r="381" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B381" s="28" t="s">
+        <v>282</v>
+      </c>
+      <c r="C381" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B382" s="28" t="s">
+        <v>283</v>
+      </c>
+      <c r="C382" s="8">
+        <v>1</v>
       </c>
     </row>
     <row r="383" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B383" s="28" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="C383" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="384" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B384" s="28" t="s">
-        <v>292</v>
-      </c>
-      <c r="C384" s="8">
-        <v>1.2</v>
-      </c>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B384" s="28"/>
     </row>
     <row r="385" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B385" s="28" t="s">
-        <v>293</v>
-      </c>
-      <c r="C385" s="8">
-        <v>0.8</v>
+      <c r="A385" s="36" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="386" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B386" s="28" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="C386" s="8">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="387" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B387" s="28" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="C387" s="8">
         <v>1.5</v>
       </c>
     </row>
-    <row r="388" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="388" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B388" s="28" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="C388" s="8">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="389" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B389" s="28" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="C389" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="390" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B390" s="28"/>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B390" s="28" t="s">
+        <v>289</v>
+      </c>
+      <c r="C390" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="391" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A391" s="36" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="392" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B392" s="28" t="s">
-        <v>298</v>
-      </c>
-      <c r="C392" s="8">
-        <v>1.2</v>
-      </c>
+      <c r="B391" s="28" t="s">
+        <v>290</v>
+      </c>
+      <c r="C391" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B392" s="28"/>
     </row>
     <row r="393" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B393" s="28" t="s">
-        <v>299</v>
-      </c>
-      <c r="C393" s="8">
-        <v>1</v>
+      <c r="A393" s="36" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="394" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B394" s="28" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="C394" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="395" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="395" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B395" s="28" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="C395" s="8">
         <v>1.2</v>
@@ -7087,380 +7180,390 @@
     </row>
     <row r="396" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B396" s="28" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="C396" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="397" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="397" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B397" s="28" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="C397" s="8">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="398" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B398" s="28" t="s">
+        <v>295</v>
+      </c>
+      <c r="C398" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B399" s="28" t="s">
+        <v>296</v>
+      </c>
+      <c r="C399" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="400" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B400" s="28" t="s">
+        <v>297</v>
+      </c>
+      <c r="C400" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="401" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B401" s="28"/>
+    </row>
+    <row r="402" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A402" s="36" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="403" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B403" s="28" t="s">
+        <v>298</v>
+      </c>
+      <c r="C403" s="8">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="404" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B404" s="28" t="s">
+        <v>299</v>
+      </c>
+      <c r="C404" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="405" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B405" s="28" t="s">
+        <v>300</v>
+      </c>
+      <c r="C405" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B406" s="28" t="s">
+        <v>301</v>
+      </c>
+      <c r="C406" s="8">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="407" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B407" s="28" t="s">
+        <v>302</v>
+      </c>
+      <c r="C407" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="408" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B408" s="28" t="s">
+        <v>303</v>
+      </c>
+      <c r="C408" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B409" s="28" t="s">
         <v>304</v>
       </c>
-      <c r="C398" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="399" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B399" s="28"/>
-    </row>
-    <row r="400" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A400" s="36" t="s">
+      <c r="C409" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B410" s="28"/>
+    </row>
+    <row r="411" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A411" s="36" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="401" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B401" s="28" t="s">
+    <row r="412" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B412" s="28" t="s">
         <v>305</v>
       </c>
-      <c r="C401" s="8">
+      <c r="C412" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="402" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B402" s="28" t="s">
+    <row r="413" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B413" s="28" t="s">
         <v>306</v>
       </c>
-      <c r="C402" s="8">
+      <c r="C413" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="403" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B403" s="28" t="s">
+    <row r="414" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B414" s="28" t="s">
         <v>307</v>
       </c>
-      <c r="C403" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="404" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B404" s="28" t="s">
+      <c r="C414" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B415" s="28" t="s">
         <v>308</v>
       </c>
-      <c r="C404" s="8">
+      <c r="C415" s="8">
         <v>0.8</v>
       </c>
     </row>
-    <row r="405" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B405" s="28" t="s">
+    <row r="416" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B416" s="28" t="s">
         <v>309</v>
       </c>
-      <c r="C405" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="406" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B406" s="28"/>
-      <c r="D406" s="14"/>
-      <c r="E406" s="14"/>
-    </row>
-    <row r="407" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A407" s="29" t="s">
+      <c r="C416" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="417" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B417" s="28"/>
+      <c r="D417" s="14"/>
+      <c r="E417" s="14"/>
+    </row>
+    <row r="418" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A418" s="29" t="s">
         <v>475</v>
       </c>
-      <c r="B407" s="31" t="s">
+      <c r="B418" s="31" t="s">
         <v>502</v>
       </c>
-      <c r="C407" s="14">
+      <c r="C418" s="14">
         <v>1.2</v>
       </c>
-      <c r="D407" s="14">
+      <c r="D418" s="14">
         <v>0.8</v>
       </c>
-      <c r="E407" s="14"/>
-    </row>
-    <row r="408" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A408" s="16"/>
-      <c r="B408" s="31" t="s">
+      <c r="E418" s="14"/>
+    </row>
+    <row r="419" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A419" s="16"/>
+      <c r="B419" s="31" t="s">
         <v>465</v>
       </c>
-      <c r="C408" s="14">
+      <c r="C419" s="14">
         <v>1.2</v>
       </c>
-      <c r="D408" s="14">
+      <c r="D419" s="14">
         <v>0.8</v>
       </c>
-      <c r="E408" s="14"/>
-    </row>
-    <row r="409" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A409" s="16"/>
-      <c r="B409" s="31" t="s">
+      <c r="E419" s="14"/>
+    </row>
+    <row r="420" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A420" s="16"/>
+      <c r="B420" s="31" t="s">
         <v>466</v>
       </c>
-      <c r="C409" s="14">
+      <c r="C420" s="14">
         <v>0.8</v>
       </c>
-      <c r="D409" s="14">
+      <c r="D420" s="14">
         <v>0.5</v>
       </c>
-      <c r="E409" s="14"/>
-    </row>
-    <row r="410" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A410" s="16"/>
-      <c r="B410" s="31" t="s">
+      <c r="E420" s="14"/>
+    </row>
+    <row r="421" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A421" s="16"/>
+      <c r="B421" s="31" t="s">
         <v>467</v>
       </c>
-      <c r="C410" s="14">
-        <v>1</v>
-      </c>
-      <c r="D410" s="14">
-        <v>1</v>
-      </c>
-      <c r="E410" s="14"/>
-    </row>
-    <row r="411" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A411" s="16"/>
-      <c r="B411" s="31" t="s">
+      <c r="C421" s="14">
+        <v>1</v>
+      </c>
+      <c r="D421" s="14">
+        <v>1</v>
+      </c>
+      <c r="E421" s="14"/>
+    </row>
+    <row r="422" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A422" s="16"/>
+      <c r="B422" s="31" t="s">
         <v>468</v>
       </c>
-      <c r="C411" s="14">
+      <c r="C422" s="14">
         <v>2</v>
       </c>
-      <c r="D411" s="14">
+      <c r="D422" s="14">
         <v>1.8</v>
       </c>
-      <c r="E411" s="14"/>
-    </row>
-    <row r="412" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A412" s="16"/>
-      <c r="B412" s="31" t="s">
+      <c r="E422" s="14"/>
+    </row>
+    <row r="423" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A423" s="16"/>
+      <c r="B423" s="31" t="s">
         <v>503</v>
       </c>
-      <c r="C412" s="14">
+      <c r="C423" s="14">
         <v>1.2</v>
       </c>
-      <c r="D412" s="14">
-        <v>1</v>
-      </c>
-      <c r="E412" s="14"/>
-    </row>
-    <row r="413" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A413" s="16"/>
-      <c r="B413" s="31" t="s">
+      <c r="D423" s="14">
+        <v>1</v>
+      </c>
+      <c r="E423" s="14"/>
+    </row>
+    <row r="424" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A424" s="16"/>
+      <c r="B424" s="31" t="s">
         <v>469</v>
       </c>
-      <c r="C413" s="14">
-        <v>1</v>
-      </c>
-      <c r="D413" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="E413" s="14"/>
-    </row>
-    <row r="414" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A414" s="16"/>
-      <c r="B414" s="31" t="s">
+      <c r="C424" s="14">
+        <v>1</v>
+      </c>
+      <c r="D424" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E424" s="14"/>
+    </row>
+    <row r="425" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A425" s="16"/>
+      <c r="B425" s="31" t="s">
         <v>470</v>
       </c>
-      <c r="C414" s="14">
+      <c r="C425" s="14">
         <v>2</v>
       </c>
-      <c r="D414" s="14">
+      <c r="D425" s="14">
         <v>2</v>
       </c>
-      <c r="E414" s="14"/>
-    </row>
-    <row r="415" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A415" s="16"/>
-      <c r="B415" s="31" t="s">
+      <c r="E425" s="14"/>
+    </row>
+    <row r="426" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A426" s="16"/>
+      <c r="B426" s="31" t="s">
         <v>471</v>
       </c>
-      <c r="C415" s="14">
+      <c r="C426" s="14">
         <v>2</v>
       </c>
-      <c r="D415" s="14">
+      <c r="D426" s="14">
         <v>2</v>
       </c>
-      <c r="E415" s="14"/>
-    </row>
-    <row r="416" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A416" s="16"/>
-      <c r="B416" s="31" t="s">
+      <c r="E426" s="14"/>
+    </row>
+    <row r="427" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A427" s="16"/>
+      <c r="B427" s="31" t="s">
         <v>472</v>
       </c>
-      <c r="C416" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D416" s="14">
+      <c r="C427" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D427" s="14">
         <v>1.8</v>
       </c>
-      <c r="E416" s="14"/>
-    </row>
-    <row r="417" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A417" s="16"/>
-      <c r="B417" s="31" t="s">
+      <c r="E427" s="14"/>
+    </row>
+    <row r="428" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A428" s="16"/>
+      <c r="B428" s="31" t="s">
         <v>473</v>
       </c>
-      <c r="C417" s="14">
+      <c r="C428" s="14">
         <v>2.5</v>
       </c>
-      <c r="D417" s="14">
+      <c r="D428" s="14">
         <v>2.5</v>
       </c>
-      <c r="E417" s="14"/>
-    </row>
-    <row r="418" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A418" s="16"/>
-      <c r="B418" s="37" t="s">
+      <c r="E428" s="14"/>
+    </row>
+    <row r="429" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A429" s="16"/>
+      <c r="B429" s="37" t="s">
         <v>474</v>
       </c>
-      <c r="C418" s="8">
-        <v>1.5</v>
-      </c>
-      <c r="D418" s="14">
-        <v>1</v>
-      </c>
-      <c r="E418" s="14"/>
-    </row>
-    <row r="419" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A419" s="16"/>
-      <c r="B419" s="8" t="s">
+      <c r="C429" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="D429" s="14">
+        <v>1</v>
+      </c>
+      <c r="E429" s="14"/>
+    </row>
+    <row r="430" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A430" s="16"/>
+      <c r="B430" s="8" t="s">
         <v>498</v>
       </c>
-      <c r="C419" s="8">
-        <v>1.5</v>
-      </c>
-      <c r="D419" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="E419" s="14"/>
-    </row>
-    <row r="420" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A420" s="16"/>
-      <c r="B420" s="8" t="s">
+      <c r="C430" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="D430" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E430" s="14"/>
+    </row>
+    <row r="431" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A431" s="16"/>
+      <c r="B431" s="8" t="s">
         <v>499</v>
       </c>
-      <c r="C420" s="8">
-        <v>1</v>
-      </c>
-      <c r="D420" s="8">
+      <c r="C431" s="8">
+        <v>1</v>
+      </c>
+      <c r="D431" s="8">
         <v>0.8</v>
       </c>
     </row>
-    <row r="421" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B421" s="8" t="s">
+    <row r="432" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B432" s="8" t="s">
         <v>500</v>
       </c>
-      <c r="C421" s="8">
-        <v>1</v>
-      </c>
-      <c r="D421" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="422" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A422" s="36" t="s">
+      <c r="C432" s="8">
+        <v>1</v>
+      </c>
+      <c r="D432" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="433" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A433" s="36" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="423" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B423" s="28" t="s">
+    <row r="434" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B434" s="28" t="s">
         <v>310</v>
       </c>
-      <c r="C423" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="424" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B424" s="28" t="s">
+      <c r="C434" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="435" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B435" s="28" t="s">
         <v>311</v>
       </c>
-      <c r="C424" s="8">
+      <c r="C435" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="425" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A425" s="26" t="s">
+    <row r="436" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A436" s="26" t="s">
         <v>447</v>
       </c>
-      <c r="B425" s="28" t="s">
+      <c r="B436" s="28" t="s">
         <v>312</v>
       </c>
-      <c r="C425" s="8">
+      <c r="C436" s="8">
         <v>1.2</v>
-      </c>
-    </row>
-    <row r="426" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B426" s="28" t="s">
-        <v>313</v>
-      </c>
-      <c r="C426" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="427" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B427" s="28" t="s">
-        <v>314</v>
-      </c>
-      <c r="C427" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="428" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B428" s="28" t="s">
-        <v>315</v>
-      </c>
-      <c r="C428" s="8">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="429" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B429" s="28" t="s">
-        <v>316</v>
-      </c>
-      <c r="C429" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="430" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B430" s="28" t="s">
-        <v>317</v>
-      </c>
-      <c r="C430" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="431" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B431" s="28" t="s">
-        <v>318</v>
-      </c>
-      <c r="C431" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="432" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B432" s="28" t="s">
-        <v>319</v>
-      </c>
-      <c r="C432" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="433" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B433" s="28"/>
-    </row>
-    <row r="434" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B434" s="28"/>
-    </row>
-    <row r="435" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B435" s="28"/>
-    </row>
-    <row r="436" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A436" s="36" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="437" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B437" s="28" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="C437" s="8">
         <v>2</v>
@@ -7468,39 +7571,39 @@
     </row>
     <row r="438" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B438" s="28" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="C438" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="439" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="439" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B439" s="28" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="C439" s="8">
-        <v>3</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="440" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B440" s="28" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="C440" s="8">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="441" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="441" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B441" s="28" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="C441" s="8">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="442" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B442" s="28" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="C442" s="8">
         <v>1</v>
@@ -7508,7 +7611,7 @@
     </row>
     <row r="443" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B443" s="28" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="C443" s="8">
         <v>1</v>
@@ -7517,8 +7620,78 @@
     <row r="444" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B444" s="28"/>
     </row>
-    <row r="445" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A445" s="26" t="s">
+    <row r="445" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B445" s="28"/>
+    </row>
+    <row r="446" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B446" s="28"/>
+    </row>
+    <row r="447" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A447" s="36" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="448" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B448" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="C448" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="449" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B449" s="28" t="s">
+        <v>321</v>
+      </c>
+      <c r="C449" s="8">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="450" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B450" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="C450" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="451" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B451" s="28" t="s">
+        <v>323</v>
+      </c>
+      <c r="C451" s="8">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="452" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B452" s="28" t="s">
+        <v>324</v>
+      </c>
+      <c r="C452" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="453" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B453" s="28" t="s">
+        <v>325</v>
+      </c>
+      <c r="C453" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="454" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B454" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="C454" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="455" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B455" s="28"/>
+    </row>
+    <row r="456" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A456" s="26" t="s">
         <v>447</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: clarify 4 agents vs technical nodes
</commit_message>
<xml_diff>
--- a/project/requisitos_backlog.xlsx
+++ b/project/requisitos_backlog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/erp-fraud-data-TFG/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31BC9D80-3BDB-6345-A51B-E7804F2BCBD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6170307C-5A4C-2E4C-911A-2126ED0E1B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUISITOS" sheetId="1" r:id="rId1"/>
@@ -1685,7 +1685,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1738,6 +1738,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -1779,7 +1785,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1909,6 +1915,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2576,28 +2597,28 @@
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
     </row>
-    <row r="17" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:9" s="49" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+      <c r="A17" s="45" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="46" t="s">
         <v>49</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="47">
         <v>8</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="40"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
+      <c r="E17" s="47" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>81</v>
+      </c>
+      <c r="G17" s="48"/>
+      <c r="H17" s="47"/>
+      <c r="I17" s="47"/>
     </row>
     <row r="18" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="20" t="s">
@@ -3194,7 +3215,7 @@
     <col min="6" max="16384" width="8.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>93</v>
       </c>
@@ -4894,7 +4915,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="181" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B181" s="28" t="s">
         <v>233</v>
       </c>
@@ -4927,7 +4948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B184" s="28" t="s">
         <v>236</v>
       </c>
@@ -4957,7 +4978,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="187" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B187" s="28" t="s">
         <v>239</v>
       </c>
@@ -4994,7 +5015,7 @@
       </c>
       <c r="E189" s="14"/>
     </row>
-    <row r="190" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A190" s="14"/>
       <c r="B190" s="28" t="s">
         <v>507</v>

</xml_diff>

<commit_message>
docs+graph: clarify integration tests and add fraud tree taxonomy
</commit_message>
<xml_diff>
--- a/project/requisitos_backlog.xlsx
+++ b/project/requisitos_backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/erp-fraud-data-TFG/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6170307C-5A4C-2E4C-911A-2126ED0E1B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6188DC8E-0774-D94B-8F89-CE31232806A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REQUISITOS" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="642" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="525">
   <si>
     <t>User story</t>
   </si>
@@ -1606,6 +1606,9 @@
   </si>
   <si>
     <t xml:space="preserve"> RF14b-11: Ejecutar verificación de criterios de aceptación y guardar evidencia (artefactos + enlace de traza LangSmith +</t>
+  </si>
+  <si>
+    <t>RF15-11: Actualizar proyecto para que fraud type proceda de documentación oficial</t>
   </si>
 </sst>
 </file>
@@ -3204,7 +3207,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:E456"/>
+  <dimension ref="A2:E457"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="71.33203125" style="26" bestFit="1" customWidth="1"/>
@@ -5958,98 +5961,98 @@
     </row>
     <row r="267" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267" s="16"/>
-      <c r="B267" s="28"/>
-      <c r="C267" s="14"/>
-      <c r="D267" s="14"/>
+      <c r="B267" s="28" t="s">
+        <v>524</v>
+      </c>
+      <c r="C267" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D267" s="14">
+        <v>1.5</v>
+      </c>
       <c r="E267" s="14"/>
     </row>
-    <row r="268" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A268" s="29" t="s">
+    <row r="268" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A268" s="16"/>
+      <c r="B268" s="28"/>
+      <c r="C268" s="14"/>
+      <c r="D268" s="14"/>
+      <c r="E268" s="14"/>
+    </row>
+    <row r="269" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A269" s="29" t="s">
         <v>358</v>
       </c>
-      <c r="B268" s="28" t="s">
+      <c r="B269" s="28" t="s">
         <v>394</v>
       </c>
-      <c r="C268" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D268" s="14">
-        <v>1</v>
-      </c>
-      <c r="E268" s="14"/>
-    </row>
-    <row r="269" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A269" s="16"/>
-      <c r="B269" s="28" t="s">
+      <c r="C269" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D269" s="14">
+        <v>1</v>
+      </c>
+      <c r="E269" s="14"/>
+    </row>
+    <row r="270" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A270" s="16"/>
+      <c r="B270" s="28" t="s">
         <v>395</v>
       </c>
-      <c r="C269" s="14">
-        <v>1</v>
-      </c>
-      <c r="D269" s="14">
-        <v>1</v>
-      </c>
-      <c r="E269" s="14"/>
-    </row>
-    <row r="270" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A270" s="19"/>
-      <c r="B270" s="31" t="s">
+      <c r="C270" s="14">
+        <v>1</v>
+      </c>
+      <c r="D270" s="14">
+        <v>1</v>
+      </c>
+      <c r="E270" s="14"/>
+    </row>
+    <row r="271" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A271" s="19"/>
+      <c r="B271" s="31" t="s">
         <v>396</v>
       </c>
-      <c r="C270" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D270" s="14">
+      <c r="C271" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D271" s="14">
         <v>1.2</v>
-      </c>
-      <c r="E270" s="14"/>
-    </row>
-    <row r="271" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A271" s="16"/>
-      <c r="B271" s="28" t="s">
-        <v>397</v>
-      </c>
-      <c r="C271" s="14">
-        <v>2</v>
-      </c>
-      <c r="D271" s="14">
-        <v>1.8</v>
       </c>
       <c r="E271" s="14"/>
     </row>
     <row r="272" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A272" s="16"/>
       <c r="B272" s="28" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C272" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D272" s="14">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E272" s="14"/>
     </row>
     <row r="273" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A273" s="16"/>
       <c r="B273" s="28" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C273" s="14">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="D273" s="14">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E273" s="14"/>
     </row>
     <row r="274" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A274" s="16"/>
       <c r="B274" s="28" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C274" s="14">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D274" s="14">
         <v>2</v>
@@ -6059,288 +6062,288 @@
     <row r="275" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A275" s="16"/>
       <c r="B275" s="28" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C275" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D275" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E275" s="14"/>
     </row>
     <row r="276" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A276" s="16"/>
       <c r="B276" s="28" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C276" s="14">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="D276" s="14">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="E276" s="14"/>
     </row>
     <row r="277" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A277" s="16"/>
       <c r="B277" s="28" t="s">
-        <v>480</v>
+        <v>402</v>
       </c>
       <c r="C277" s="14">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="D277" s="14">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="E277" s="14"/>
     </row>
     <row r="278" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A278" s="16"/>
       <c r="B278" s="28" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C278" s="14">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="D278" s="14">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E278" s="14"/>
     </row>
     <row r="279" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A279" s="16"/>
       <c r="B279" s="28" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C279" s="14">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="D279" s="14">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E279" s="14"/>
     </row>
     <row r="280" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A280" s="16"/>
-      <c r="B280" s="28"/>
-      <c r="C280" s="14"/>
-      <c r="D280" s="14"/>
+      <c r="B280" s="28" t="s">
+        <v>482</v>
+      </c>
+      <c r="C280" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="D280" s="14">
+        <v>0.5</v>
+      </c>
       <c r="E280" s="14"/>
     </row>
     <row r="281" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A281" s="16" t="s">
-        <v>447</v>
-      </c>
+      <c r="A281" s="16"/>
       <c r="B281" s="28"/>
       <c r="C281" s="14"/>
       <c r="D281" s="14"/>
       <c r="E281" s="14"/>
     </row>
-    <row r="282" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A282" s="29" t="s">
+    <row r="282" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A282" s="16" t="s">
+        <v>447</v>
+      </c>
+      <c r="B282" s="28"/>
+      <c r="C282" s="14"/>
+      <c r="D282" s="14"/>
+      <c r="E282" s="14"/>
+    </row>
+    <row r="283" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A283" s="29" t="s">
         <v>361</v>
       </c>
-      <c r="B282" s="28" t="s">
+      <c r="B283" s="28" t="s">
         <v>403</v>
-      </c>
-      <c r="C282" s="14">
-        <v>2</v>
-      </c>
-      <c r="D282" s="14">
-        <v>2.5</v>
-      </c>
-      <c r="E282" s="14"/>
-    </row>
-    <row r="283" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A283" s="19"/>
-      <c r="B283" s="31" t="s">
-        <v>404</v>
       </c>
       <c r="C283" s="14">
         <v>2</v>
       </c>
       <c r="D283" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="E283" s="14"/>
+    </row>
+    <row r="284" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A284" s="19"/>
+      <c r="B284" s="31" t="s">
+        <v>404</v>
+      </c>
+      <c r="C284" s="14">
+        <v>2</v>
+      </c>
+      <c r="D284" s="14">
         <v>3</v>
-      </c>
-      <c r="E283" s="14"/>
-    </row>
-    <row r="284" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A284" s="16"/>
-      <c r="B284" s="28" t="s">
-        <v>405</v>
-      </c>
-      <c r="C284" s="14">
-        <v>2.5</v>
-      </c>
-      <c r="D284" s="14">
-        <v>3.8</v>
       </c>
       <c r="E284" s="14"/>
     </row>
     <row r="285" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A285" s="16"/>
       <c r="B285" s="28" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C285" s="14">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="D285" s="14">
-        <v>2</v>
+        <v>3.8</v>
       </c>
       <c r="E285" s="14"/>
     </row>
-    <row r="286" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A286" s="16"/>
       <c r="B286" s="28" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C286" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D286" s="14">
         <v>2</v>
       </c>
-      <c r="D286" s="14">
-        <v>2.2000000000000002</v>
-      </c>
       <c r="E286" s="14"/>
     </row>
-    <row r="287" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A287" s="16"/>
       <c r="B287" s="28" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C287" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D287" s="14">
-        <v>1.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E287" s="14"/>
     </row>
-    <row r="288" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A288" s="16"/>
       <c r="B288" s="28" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C288" s="14">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D288" s="14">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="E288" s="14"/>
     </row>
-    <row r="289" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A289" s="16"/>
       <c r="B289" s="28" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C289" s="14">
         <v>2</v>
       </c>
       <c r="D289" s="14">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="E289" s="14"/>
     </row>
-    <row r="290" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A290" s="16"/>
       <c r="B290" s="28" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C290" s="14">
         <v>2</v>
       </c>
       <c r="D290" s="14">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="E290" s="14"/>
     </row>
     <row r="291" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A291" s="16"/>
       <c r="B291" s="28" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C291" s="14">
         <v>2</v>
       </c>
       <c r="D291" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="E291" s="14"/>
+    </row>
+    <row r="292" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A292" s="16"/>
+      <c r="B292" s="28" t="s">
+        <v>412</v>
+      </c>
+      <c r="C292" s="14">
         <v>2</v>
       </c>
-      <c r="E291" s="14"/>
-    </row>
-    <row r="292" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A292" s="19"/>
-      <c r="B292" s="31" t="s">
+      <c r="D292" s="14">
+        <v>2</v>
+      </c>
+      <c r="E292" s="14"/>
+    </row>
+    <row r="293" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A293" s="19"/>
+      <c r="B293" s="31" t="s">
         <v>413</v>
       </c>
-      <c r="C292" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D292" s="14">
+      <c r="C293" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D293" s="14">
         <v>1.2</v>
-      </c>
-      <c r="E292" s="14"/>
-    </row>
-    <row r="293" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A293" s="16"/>
-      <c r="B293" s="28" t="s">
-        <v>414</v>
-      </c>
-      <c r="C293" s="14">
-        <v>1</v>
-      </c>
-      <c r="D293" s="14">
-        <v>1</v>
       </c>
       <c r="E293" s="14"/>
     </row>
     <row r="294" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A294" s="16"/>
       <c r="B294" s="28" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C294" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D294" s="14">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="E294" s="14"/>
     </row>
     <row r="295" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A295" s="16"/>
       <c r="B295" s="28" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C295" s="14">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="D295" s="14">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="E295" s="14"/>
     </row>
     <row r="296" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A296" s="16"/>
       <c r="B296" s="28" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C296" s="14">
         <v>1.5</v>
       </c>
       <c r="D296" s="14">
-        <v>1.5</v>
+        <v>2.8</v>
       </c>
       <c r="E296" s="14"/>
     </row>
     <row r="297" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A297" s="16"/>
       <c r="B297" s="28" t="s">
-        <v>489</v>
-      </c>
-      <c r="C297" s="8">
-        <v>2</v>
+        <v>417</v>
+      </c>
+      <c r="C297" s="14">
+        <v>1.5</v>
       </c>
       <c r="D297" s="14">
         <v>1.5</v>
@@ -6350,20 +6353,20 @@
     <row r="298" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A298" s="16"/>
       <c r="B298" s="28" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C298" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D298" s="14">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E298" s="14"/>
     </row>
     <row r="299" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A299" s="16"/>
       <c r="B299" s="28" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C299" s="8">
         <v>1</v>
@@ -6374,174 +6377,176 @@
       <c r="E299" s="14"/>
     </row>
     <row r="300" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A300" s="16" t="s">
+      <c r="A300" s="16"/>
+      <c r="B300" s="28" t="s">
+        <v>491</v>
+      </c>
+      <c r="C300" s="8">
+        <v>1</v>
+      </c>
+      <c r="D300" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="E300" s="14"/>
+    </row>
+    <row r="301" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A301" s="16" t="s">
         <v>447</v>
       </c>
-      <c r="B300" s="28"/>
-      <c r="C300" s="14"/>
-      <c r="D300" s="14"/>
-      <c r="E300" s="14"/>
-    </row>
-    <row r="301" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A301" s="29" t="s">
+      <c r="B301" s="28"/>
+      <c r="C301" s="14"/>
+      <c r="D301" s="14"/>
+      <c r="E301" s="14"/>
+    </row>
+    <row r="302" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A302" s="29" t="s">
         <v>364</v>
       </c>
-      <c r="B301" s="18" t="s">
+      <c r="B302" s="18" t="s">
         <v>418</v>
       </c>
-      <c r="C301" s="14">
+      <c r="C302" s="14">
         <v>0.8</v>
       </c>
-      <c r="D301" s="14">
+      <c r="D302" s="14">
         <v>0.5</v>
-      </c>
-      <c r="E301" s="14"/>
-    </row>
-    <row r="302" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A302" s="16"/>
-      <c r="B302" s="18" t="s">
-        <v>419</v>
-      </c>
-      <c r="C302" s="14">
-        <v>2</v>
-      </c>
-      <c r="D302" s="14">
-        <v>1.8</v>
       </c>
       <c r="E302" s="14"/>
     </row>
     <row r="303" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A303" s="16"/>
       <c r="B303" s="18" t="s">
+        <v>419</v>
+      </c>
+      <c r="C303" s="14">
+        <v>2</v>
+      </c>
+      <c r="D303" s="14">
+        <v>1.8</v>
+      </c>
+      <c r="E303" s="14"/>
+    </row>
+    <row r="304" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A304" s="16"/>
+      <c r="B304" s="18" t="s">
         <v>420</v>
       </c>
-      <c r="C303" s="14">
+      <c r="C304" s="14">
         <v>1.2</v>
       </c>
-      <c r="D303" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="E303" s="14"/>
-    </row>
-    <row r="304" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A304" s="19"/>
-      <c r="B304" s="14" t="s">
+      <c r="D304" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E304" s="14"/>
+    </row>
+    <row r="305" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A305" s="19"/>
+      <c r="B305" s="14" t="s">
         <v>421</v>
       </c>
-      <c r="C304" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D304" s="14">
+      <c r="C305" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D305" s="14">
         <v>1.8</v>
-      </c>
-      <c r="E304" s="14"/>
-    </row>
-    <row r="305" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A305" s="16"/>
-      <c r="B305" s="18" t="s">
-        <v>422</v>
-      </c>
-      <c r="C305" s="14">
-        <v>2.5</v>
-      </c>
-      <c r="D305" s="14">
-        <v>2.5</v>
       </c>
       <c r="E305" s="14"/>
     </row>
     <row r="306" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A306" s="16"/>
       <c r="B306" s="18" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C306" s="14">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D306" s="14">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E306" s="14"/>
     </row>
     <row r="307" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A307" s="16"/>
       <c r="B307" s="18" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C307" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D307" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E307" s="14"/>
     </row>
     <row r="308" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A308" s="16"/>
       <c r="B308" s="18" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C308" s="14">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="D308" s="14">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="E308" s="14"/>
     </row>
     <row r="309" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A309" s="16"/>
       <c r="B309" s="18" t="s">
-        <v>504</v>
+        <v>425</v>
       </c>
       <c r="C309" s="14">
-        <v>1.2</v>
+        <v>3</v>
       </c>
       <c r="D309" s="14">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="E309" s="14"/>
     </row>
     <row r="310" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A310" s="16"/>
       <c r="B310" s="18" t="s">
-        <v>426</v>
+        <v>504</v>
       </c>
       <c r="C310" s="14">
         <v>1.2</v>
       </c>
       <c r="D310" s="14">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E310" s="14"/>
     </row>
     <row r="311" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A311" s="16"/>
       <c r="B311" s="18" t="s">
-        <v>492</v>
+        <v>426</v>
       </c>
       <c r="C311" s="14">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="D311" s="14">
         <v>1</v>
       </c>
       <c r="E311" s="14"/>
     </row>
-    <row r="312" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A312" s="16"/>
       <c r="B312" s="18" t="s">
+        <v>492</v>
+      </c>
+      <c r="C312" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D312" s="14">
+        <v>1</v>
+      </c>
+      <c r="E312" s="14"/>
+    </row>
+    <row r="313" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A313" s="16"/>
+      <c r="B313" s="18" t="s">
         <v>493</v>
-      </c>
-      <c r="C312" s="14">
-        <v>1</v>
-      </c>
-      <c r="D312" s="8">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="313" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B313" s="18" t="s">
-        <v>494</v>
       </c>
       <c r="C313" s="14">
         <v>1</v>
@@ -6550,173 +6555,171 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="314" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A314" s="36" t="s">
+    <row r="314" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B314" s="18" t="s">
+        <v>494</v>
+      </c>
+      <c r="C314" s="14">
+        <v>1</v>
+      </c>
+      <c r="D314" s="8">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="315" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A315" s="36" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="315" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B315" s="28" t="s">
+    <row r="316" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B316" s="28" t="s">
         <v>240</v>
       </c>
-      <c r="C315" s="8">
+      <c r="C316" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="316" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B316" s="28" t="s">
+    <row r="317" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B317" s="28" t="s">
         <v>241</v>
       </c>
-      <c r="C316" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="317" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B317" s="28" t="s">
-        <v>242</v>
-      </c>
       <c r="C317" s="8">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="318" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B318" s="28" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C318" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="319" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B319" s="28" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C319" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="320" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B320" s="28" t="s">
+        <v>244</v>
+      </c>
+      <c r="C320" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B321" s="28" t="s">
         <v>245</v>
       </c>
-      <c r="C320" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="321" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B321" s="28" t="s">
+      <c r="C321" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="322" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B322" s="28" t="s">
         <v>246</v>
       </c>
-      <c r="C321" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="322" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B322" s="28" t="s">
+      <c r="C322" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B323" s="28" t="s">
         <v>247</v>
       </c>
-      <c r="C322" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B323" s="28"/>
-    </row>
-    <row r="324" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A324" s="36" t="s">
+      <c r="C323" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B324" s="28"/>
+    </row>
+    <row r="325" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A325" s="36" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="325" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B325" s="28" t="s">
-        <v>248</v>
-      </c>
-      <c r="C325" s="8">
-        <v>1.2</v>
       </c>
     </row>
     <row r="326" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B326" s="28" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C326" s="8">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="327" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B327" s="28" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C327" s="8">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="328" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B328" s="28" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C328" s="8">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="329" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B329" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="C329" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="330" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B330" s="28" t="s">
         <v>252</v>
       </c>
-      <c r="C329" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="330" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B330" s="28" t="s">
+      <c r="C330" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="331" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="B331" s="28" t="s">
         <v>253</v>
       </c>
-      <c r="C330" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="331" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B331" s="28" t="s">
+      <c r="C331" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="332" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B332" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="C331" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B332" s="28"/>
-    </row>
-    <row r="333" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A333" s="29" t="s">
+      <c r="C332" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B333" s="28"/>
+    </row>
+    <row r="334" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A334" s="29" t="s">
         <v>367</v>
       </c>
-      <c r="B333" s="28" t="s">
+      <c r="B334" s="28" t="s">
         <v>434</v>
       </c>
-      <c r="C333" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D333" s="14">
+      <c r="C334" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D334" s="14">
         <v>1.2</v>
       </c>
-      <c r="E333" s="14"/>
-    </row>
-    <row r="334" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B334" s="28" t="s">
+      <c r="E334" s="14"/>
+    </row>
+    <row r="335" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B335" s="28" t="s">
         <v>435</v>
-      </c>
-      <c r="C334" s="14">
-        <v>1.5</v>
-      </c>
-      <c r="D334" s="14">
-        <v>2</v>
-      </c>
-      <c r="E334" s="14"/>
-    </row>
-    <row r="335" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A335" s="16"/>
-      <c r="B335" s="28" t="s">
-        <v>436</v>
       </c>
       <c r="C335" s="14">
         <v>1.5</v>
@@ -6729,101 +6732,101 @@
     <row r="336" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A336" s="16"/>
       <c r="B336" s="28" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C336" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D336" s="14">
         <v>2</v>
-      </c>
-      <c r="D336" s="14">
-        <v>2.2000000000000002</v>
       </c>
       <c r="E336" s="14"/>
     </row>
     <row r="337" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A337" s="16"/>
       <c r="B337" s="28" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C337" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D337" s="14">
-        <v>1.5</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E337" s="14"/>
     </row>
     <row r="338" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A338" s="16"/>
       <c r="B338" s="28" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C338" s="14">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="D338" s="14">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E338" s="14"/>
     </row>
     <row r="339" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A339" s="16"/>
       <c r="B339" s="28" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C339" s="14">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="D339" s="14">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E339" s="14"/>
     </row>
-    <row r="340" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A340" s="16"/>
       <c r="B340" s="28" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C340" s="14">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D340" s="14">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="E340" s="14"/>
     </row>
-    <row r="341" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A341" s="16"/>
       <c r="B341" s="28" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C341" s="14">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D341" s="14">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="E341" s="14"/>
     </row>
     <row r="342" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A342" s="16"/>
       <c r="B342" s="28" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C342" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D342" s="14">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E342" s="14"/>
     </row>
     <row r="343" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A343" s="16"/>
       <c r="B343" s="28" t="s">
-        <v>495</v>
-      </c>
-      <c r="C343" s="8">
-        <v>1.5</v>
+        <v>443</v>
+      </c>
+      <c r="C343" s="14">
+        <v>1</v>
       </c>
       <c r="D343" s="14">
         <v>1</v>
@@ -6833,57 +6836,62 @@
     <row r="344" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A344" s="16"/>
       <c r="B344" s="28" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C344" s="8">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D344" s="14">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E344" s="14"/>
     </row>
     <row r="345" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A345" s="16"/>
       <c r="B345" s="28" t="s">
+        <v>496</v>
+      </c>
+      <c r="C345" s="8">
+        <v>1</v>
+      </c>
+      <c r="D345" s="14">
+        <v>0.8</v>
+      </c>
+      <c r="E345" s="14"/>
+    </row>
+    <row r="346" spans="1:5" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A346" s="16"/>
+      <c r="B346" s="28" t="s">
         <v>497</v>
       </c>
-      <c r="C345" s="8">
-        <v>1</v>
-      </c>
-      <c r="D345" s="8">
+      <c r="C346" s="8">
+        <v>1</v>
+      </c>
+      <c r="D346" s="8">
         <v>0.5</v>
       </c>
-      <c r="E345" s="14"/>
-    </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A346" s="16"/>
-      <c r="B346" s="28"/>
-    </row>
-    <row r="347" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A347" s="36" t="s">
+      <c r="E346" s="14"/>
+    </row>
+    <row r="347" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A347" s="16"/>
+      <c r="B347" s="28"/>
+    </row>
+    <row r="348" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A348" s="36" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="348" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="B348" s="28" t="s">
-        <v>255</v>
-      </c>
-      <c r="C348" s="8">
-        <v>1</v>
       </c>
     </row>
     <row r="349" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B349" s="28" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C349" s="8">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="350" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B350" s="28" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C350" s="8">
         <v>1.5</v>
@@ -6891,71 +6899,71 @@
     </row>
     <row r="351" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B351" s="28" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C351" s="8">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="352" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B352" s="28" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C352" s="8">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="353" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B353" s="28" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C353" s="8">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="354" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B354" s="28" t="s">
+        <v>260</v>
+      </c>
+      <c r="C354" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B355" s="28" t="s">
         <v>261</v>
       </c>
-      <c r="C354" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="355" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B355" s="28" t="s">
+      <c r="C355" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B356" s="28" t="s">
         <v>262</v>
       </c>
-      <c r="C355" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="356" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B356" s="28" t="s">
+      <c r="C356" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B357" s="28" t="s">
         <v>263</v>
       </c>
-      <c r="C356" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="357" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B357" s="28"/>
-    </row>
-    <row r="358" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A358" s="36" t="s">
+      <c r="C357" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B358" s="28"/>
+    </row>
+    <row r="359" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A359" s="36" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="359" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B359" s="28" t="s">
+    <row r="360" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B360" s="28" t="s">
         <v>264</v>
-      </c>
-      <c r="C359" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="360" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B360" s="28" t="s">
-        <v>265</v>
       </c>
       <c r="C360" s="8">
         <v>1.2</v>
@@ -6963,7 +6971,7 @@
     </row>
     <row r="361" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B361" s="28" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C361" s="8">
         <v>1.2</v>
@@ -6971,55 +6979,55 @@
     </row>
     <row r="362" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B362" s="28" t="s">
+        <v>266</v>
+      </c>
+      <c r="C362" s="8">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B363" s="28" t="s">
         <v>267</v>
       </c>
-      <c r="C362" s="8">
+      <c r="C363" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="363" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B363" s="28" t="s">
+    <row r="364" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B364" s="28" t="s">
         <v>268</v>
       </c>
-      <c r="C363" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="364" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B364" s="28" t="s">
+      <c r="C364" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B365" s="28" t="s">
         <v>269</v>
       </c>
-      <c r="C364" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="365" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B365" s="28" t="s">
+      <c r="C365" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B366" s="28" t="s">
         <v>270</v>
       </c>
-      <c r="C365" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="366" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B366" s="28"/>
-    </row>
-    <row r="367" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A367" s="36" t="s">
+      <c r="C366" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B367" s="28"/>
+    </row>
+    <row r="368" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A368" s="36" t="s">
         <v>66</v>
-      </c>
-    </row>
-    <row r="368" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B368" s="28" t="s">
-        <v>271</v>
-      </c>
-      <c r="C368" s="8">
-        <v>0.8</v>
       </c>
     </row>
     <row r="369" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B369" s="28" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C369" s="8">
         <v>0.8</v>
@@ -7027,79 +7035,79 @@
     </row>
     <row r="370" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B370" s="28" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C370" s="8">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="371" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B371" s="28" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C371" s="8">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="372" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B372" s="28" t="s">
+        <v>274</v>
+      </c>
+      <c r="C372" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B373" s="28" t="s">
         <v>275</v>
       </c>
-      <c r="C372" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="373" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B373" s="28" t="s">
+      <c r="C373" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B374" s="28" t="s">
         <v>276</v>
       </c>
-      <c r="C373" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="374" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B374" s="28" t="s">
+      <c r="C374" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B375" s="28" t="s">
         <v>277</v>
       </c>
-      <c r="C374" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="375" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B375" s="28"/>
-    </row>
-    <row r="376" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A376" s="36" t="s">
+      <c r="C375" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B376" s="28"/>
+    </row>
+    <row r="377" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A377" s="36" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="377" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B377" s="28" t="s">
+    <row r="378" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B378" s="28" t="s">
         <v>278</v>
       </c>
-      <c r="C377" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="378" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B378" s="28" t="s">
+      <c r="C378" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="379" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B379" s="28" t="s">
         <v>279</v>
       </c>
-      <c r="C378" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="379" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B379" s="28" t="s">
-        <v>280</v>
-      </c>
       <c r="C379" s="8">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="380" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B380" s="28" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C380" s="8">
         <v>1</v>
@@ -7107,47 +7115,47 @@
     </row>
     <row r="381" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B381" s="28" t="s">
+        <v>281</v>
+      </c>
+      <c r="C381" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B382" s="28" t="s">
         <v>282</v>
       </c>
-      <c r="C381" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="382" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B382" s="28" t="s">
+      <c r="C382" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B383" s="28" t="s">
         <v>283</v>
       </c>
-      <c r="C382" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="383" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B383" s="28" t="s">
+      <c r="C383" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B384" s="28" t="s">
         <v>284</v>
       </c>
-      <c r="C383" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="384" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B384" s="28"/>
-    </row>
-    <row r="385" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A385" s="36" t="s">
+      <c r="C384" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B385" s="28"/>
+    </row>
+    <row r="386" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A386" s="36" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="386" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B386" s="28" t="s">
-        <v>285</v>
-      </c>
-      <c r="C386" s="8">
-        <v>1.5</v>
       </c>
     </row>
     <row r="387" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B387" s="28" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C387" s="8">
         <v>1.5</v>
@@ -7155,71 +7163,71 @@
     </row>
     <row r="388" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B388" s="28" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C388" s="8">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="389" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B389" s="28" t="s">
+        <v>287</v>
+      </c>
+      <c r="C389" s="8">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B390" s="28" t="s">
         <v>288</v>
       </c>
-      <c r="C389" s="8">
+      <c r="C390" s="8">
         <v>0.8</v>
       </c>
     </row>
-    <row r="390" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B390" s="28" t="s">
+    <row r="391" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B391" s="28" t="s">
         <v>289</v>
       </c>
-      <c r="C390" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="391" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B391" s="28" t="s">
+      <c r="C391" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B392" s="28" t="s">
         <v>290</v>
       </c>
-      <c r="C391" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="392" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B392" s="28"/>
-    </row>
-    <row r="393" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A393" s="36" t="s">
+      <c r="C392" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="393" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B393" s="28"/>
+    </row>
+    <row r="394" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A394" s="36" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="394" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B394" s="28" t="s">
-        <v>291</v>
-      </c>
-      <c r="C394" s="8">
-        <v>1</v>
       </c>
     </row>
     <row r="395" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B395" s="28" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C395" s="8">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="396" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B396" s="28" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C396" s="8">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="397" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B397" s="28" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C397" s="8">
         <v>0.8</v>
@@ -7227,111 +7235,111 @@
     </row>
     <row r="398" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B398" s="28" t="s">
+        <v>294</v>
+      </c>
+      <c r="C398" s="8">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B399" s="28" t="s">
         <v>295</v>
       </c>
-      <c r="C398" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="399" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B399" s="28" t="s">
+      <c r="C399" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="400" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B400" s="28" t="s">
         <v>296</v>
       </c>
-      <c r="C399" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="400" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B400" s="28" t="s">
+      <c r="C400" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="401" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B401" s="28" t="s">
         <v>297</v>
       </c>
-      <c r="C400" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="401" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B401" s="28"/>
-    </row>
-    <row r="402" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A402" s="36" t="s">
+      <c r="C401" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B402" s="28"/>
+    </row>
+    <row r="403" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A403" s="36" t="s">
         <v>78</v>
-      </c>
-    </row>
-    <row r="403" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B403" s="28" t="s">
-        <v>298</v>
-      </c>
-      <c r="C403" s="8">
-        <v>1.2</v>
       </c>
     </row>
     <row r="404" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B404" s="28" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C404" s="8">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="405" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B405" s="28" t="s">
+        <v>299</v>
+      </c>
+      <c r="C405" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B406" s="28" t="s">
         <v>300</v>
       </c>
-      <c r="C405" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="406" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B406" s="28" t="s">
+      <c r="C406" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="407" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B407" s="28" t="s">
         <v>301</v>
       </c>
-      <c r="C406" s="8">
+      <c r="C407" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="407" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B407" s="28" t="s">
+    <row r="408" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B408" s="28" t="s">
         <v>302</v>
       </c>
-      <c r="C407" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="408" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B408" s="28" t="s">
+      <c r="C408" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B409" s="28" t="s">
         <v>303</v>
       </c>
-      <c r="C408" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="409" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B409" s="28" t="s">
+      <c r="C409" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B410" s="28" t="s">
         <v>304</v>
       </c>
-      <c r="C409" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="410" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B410" s="28"/>
-    </row>
-    <row r="411" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A411" s="36" t="s">
+      <c r="C410" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B411" s="28"/>
+    </row>
+    <row r="412" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A412" s="36" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="412" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B412" s="28" t="s">
+    <row r="413" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B413" s="28" t="s">
         <v>305</v>
-      </c>
-      <c r="C412" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="413" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B413" s="28" t="s">
-        <v>306</v>
       </c>
       <c r="C413" s="8">
         <v>1.2</v>
@@ -7339,52 +7347,47 @@
     </row>
     <row r="414" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="B414" s="28" t="s">
+        <v>306</v>
+      </c>
+      <c r="C414" s="8">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B415" s="28" t="s">
         <v>307</v>
       </c>
-      <c r="C414" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="415" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B415" s="28" t="s">
-        <v>308</v>
-      </c>
       <c r="C415" s="8">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="416" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B416" s="28" t="s">
+        <v>308</v>
+      </c>
+      <c r="C416" s="8">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="417" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="B417" s="28" t="s">
         <v>309</v>
       </c>
-      <c r="C416" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="417" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B417" s="28"/>
-      <c r="D417" s="14"/>
-      <c r="E417" s="14"/>
-    </row>
-    <row r="418" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A418" s="29" t="s">
+      <c r="C417" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="418" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B418" s="28"/>
+      <c r="D418" s="14"/>
+      <c r="E418" s="14"/>
+    </row>
+    <row r="419" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A419" s="29" t="s">
         <v>475</v>
       </c>
-      <c r="B418" s="31" t="s">
+      <c r="B419" s="31" t="s">
         <v>502</v>
-      </c>
-      <c r="C418" s="14">
-        <v>1.2</v>
-      </c>
-      <c r="D418" s="14">
-        <v>0.8</v>
-      </c>
-      <c r="E418" s="14"/>
-    </row>
-    <row r="419" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A419" s="16"/>
-      <c r="B419" s="31" t="s">
-        <v>465</v>
       </c>
       <c r="C419" s="14">
         <v>1.2</v>
@@ -7394,88 +7397,88 @@
       </c>
       <c r="E419" s="14"/>
     </row>
-    <row r="420" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+    <row r="420" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A420" s="16"/>
       <c r="B420" s="31" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C420" s="14">
+        <v>1.2</v>
+      </c>
+      <c r="D420" s="14">
         <v>0.8</v>
       </c>
-      <c r="D420" s="14">
-        <v>0.5</v>
-      </c>
       <c r="E420" s="14"/>
     </row>
-    <row r="421" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="421" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A421" s="16"/>
       <c r="B421" s="31" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C421" s="14">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="D421" s="14">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E421" s="14"/>
     </row>
     <row r="422" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A422" s="16"/>
       <c r="B422" s="31" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C422" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D422" s="14">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="E422" s="14"/>
     </row>
     <row r="423" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A423" s="16"/>
       <c r="B423" s="31" t="s">
-        <v>503</v>
+        <v>468</v>
       </c>
       <c r="C423" s="14">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="D423" s="14">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="E423" s="14"/>
     </row>
     <row r="424" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A424" s="16"/>
       <c r="B424" s="31" t="s">
-        <v>469</v>
+        <v>503</v>
       </c>
       <c r="C424" s="14">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="D424" s="14">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E424" s="14"/>
     </row>
     <row r="425" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A425" s="16"/>
       <c r="B425" s="31" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C425" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D425" s="14">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E425" s="14"/>
     </row>
     <row r="426" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A426" s="16"/>
       <c r="B426" s="31" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C426" s="14">
         <v>2</v>
@@ -7488,241 +7491,254 @@
     <row r="427" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A427" s="16"/>
       <c r="B427" s="31" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C427" s="14">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D427" s="14">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="E427" s="14"/>
     </row>
     <row r="428" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A428" s="16"/>
       <c r="B428" s="31" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C428" s="14">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="D428" s="14">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="E428" s="14"/>
     </row>
     <row r="429" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A429" s="16"/>
-      <c r="B429" s="37" t="s">
+      <c r="B429" s="31" t="s">
+        <v>473</v>
+      </c>
+      <c r="C429" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="D429" s="14">
+        <v>2.5</v>
+      </c>
+      <c r="E429" s="14"/>
+    </row>
+    <row r="430" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A430" s="16"/>
+      <c r="B430" s="37" t="s">
         <v>474</v>
       </c>
-      <c r="C429" s="8">
-        <v>1.5</v>
-      </c>
-      <c r="D429" s="14">
-        <v>1</v>
-      </c>
-      <c r="E429" s="14"/>
-    </row>
-    <row r="430" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A430" s="16"/>
-      <c r="B430" s="8" t="s">
-        <v>498</v>
-      </c>
       <c r="C430" s="8">
         <v>1.5</v>
       </c>
       <c r="D430" s="14">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E430" s="14"/>
     </row>
-    <row r="431" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+    <row r="431" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A431" s="16"/>
       <c r="B431" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="C431" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="D431" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="E431" s="14"/>
+    </row>
+    <row r="432" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A432" s="16"/>
+      <c r="B432" s="8" t="s">
         <v>499</v>
       </c>
-      <c r="C431" s="8">
-        <v>1</v>
-      </c>
-      <c r="D431" s="8">
+      <c r="C432" s="8">
+        <v>1</v>
+      </c>
+      <c r="D432" s="8">
         <v>0.8</v>
       </c>
     </row>
-    <row r="432" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="B432" s="8" t="s">
+    <row r="433" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B433" s="8" t="s">
         <v>500</v>
       </c>
-      <c r="C432" s="8">
-        <v>1</v>
-      </c>
-      <c r="D432" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="433" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A433" s="36" t="s">
+      <c r="C433" s="8">
+        <v>1</v>
+      </c>
+      <c r="D433" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="434" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A434" s="36" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="434" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B434" s="28" t="s">
+    <row r="435" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B435" s="28" t="s">
         <v>310</v>
       </c>
-      <c r="C434" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="435" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B435" s="28" t="s">
+      <c r="C435" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="436" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B436" s="28" t="s">
         <v>311</v>
-      </c>
-      <c r="C435" s="8">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="436" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A436" s="26" t="s">
-        <v>447</v>
-      </c>
-      <c r="B436" s="28" t="s">
-        <v>312</v>
       </c>
       <c r="C436" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="437" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+    <row r="437" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A437" s="26" t="s">
+        <v>447</v>
+      </c>
       <c r="B437" s="28" t="s">
+        <v>312</v>
+      </c>
+      <c r="C437" s="8">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="438" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B438" s="28" t="s">
         <v>313</v>
       </c>
-      <c r="C437" s="8">
+      <c r="C438" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="438" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B438" s="28" t="s">
+    <row r="439" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B439" s="28" t="s">
         <v>314</v>
       </c>
-      <c r="C438" s="8">
+      <c r="C439" s="8">
         <v>1.2</v>
       </c>
     </row>
-    <row r="439" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B439" s="28" t="s">
+    <row r="440" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B440" s="28" t="s">
         <v>315</v>
       </c>
-      <c r="C439" s="8">
+      <c r="C440" s="8">
         <v>1.8</v>
       </c>
     </row>
-    <row r="440" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B440" s="28" t="s">
+    <row r="441" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B441" s="28" t="s">
         <v>316</v>
       </c>
-      <c r="C440" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="441" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B441" s="28" t="s">
+      <c r="C441" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="442" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B442" s="28" t="s">
         <v>317</v>
       </c>
-      <c r="C441" s="8">
+      <c r="C442" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="442" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B442" s="28" t="s">
+    <row r="443" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B443" s="28" t="s">
         <v>318</v>
       </c>
-      <c r="C442" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="443" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B443" s="28" t="s">
+      <c r="C443" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="444" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="B444" s="28" t="s">
         <v>319</v>
       </c>
-      <c r="C443" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="444" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B444" s="28"/>
-    </row>
-    <row r="445" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C444" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="445" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B445" s="28"/>
     </row>
-    <row r="446" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="446" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B446" s="28"/>
     </row>
-    <row r="447" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A447" s="36" t="s">
+    <row r="447" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B447" s="28"/>
+    </row>
+    <row r="448" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A448" s="36" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="448" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B448" s="28" t="s">
+    <row r="449" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B449" s="28" t="s">
         <v>320</v>
       </c>
-      <c r="C448" s="8">
+      <c r="C449" s="8">
         <v>2</v>
-      </c>
-    </row>
-    <row r="449" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B449" s="28" t="s">
-        <v>321</v>
-      </c>
-      <c r="C449" s="8">
-        <v>1.2</v>
       </c>
     </row>
     <row r="450" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B450" s="28" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C450" s="8">
-        <v>3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="451" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B451" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="C451" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="452" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B452" s="28" t="s">
         <v>323</v>
       </c>
-      <c r="C451" s="8">
+      <c r="C452" s="8">
         <v>2.5</v>
       </c>
     </row>
-    <row r="452" spans="1:3" ht="34" x14ac:dyDescent="0.2">
-      <c r="B452" s="28" t="s">
+    <row r="453" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="B453" s="28" t="s">
         <v>324</v>
       </c>
-      <c r="C452" s="8">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="453" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="B453" s="28" t="s">
-        <v>325</v>
-      </c>
       <c r="C453" s="8">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="454" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="B454" s="28" t="s">
+        <v>325</v>
+      </c>
+      <c r="C454" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="455" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B455" s="28" t="s">
         <v>326</v>
       </c>
-      <c r="C454" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="455" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B455" s="28"/>
-    </row>
-    <row r="456" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A456" s="26" t="s">
+      <c r="C455" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="456" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B456" s="28"/>
+    </row>
+    <row r="457" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A457" s="26" t="s">
         <v>447</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RF14c closeout docs/tests and fix CI output contract
</commit_message>
<xml_diff>
--- a/project/requisitos_backlog.xlsx
+++ b/project/requisitos_backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luciasorniscaletti/Desktop/UNI/TFG/erp-fraud-data-TFG/project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0422E04-F5C0-8F43-9F81-18EFF0447C41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F59955-2D88-2C43-9BCD-1E06AEA35B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1921,7 +1921,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2091,12 +2091,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3508,7 +3502,7 @@
     <col min="5" max="16384" width="8.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="17" t="s">
         <v>87</v>
       </c>
@@ -6078,7 +6072,9 @@
       <c r="C257" s="14">
         <v>0.8</v>
       </c>
-      <c r="D257" s="14"/>
+      <c r="D257" s="14">
+        <v>1</v>
+      </c>
     </row>
     <row r="258" spans="1:4" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="16"/>
@@ -6088,7 +6084,9 @@
       <c r="C258" s="14">
         <v>1.2</v>
       </c>
-      <c r="D258" s="14"/>
+      <c r="D258" s="14">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="259" spans="1:4" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259" s="16"/>
@@ -6098,7 +6096,9 @@
       <c r="C259" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D259" s="14"/>
+      <c r="D259" s="14">
+        <v>2</v>
+      </c>
     </row>
     <row r="260" spans="1:4" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="16"/>
@@ -6108,7 +6108,9 @@
       <c r="C260" s="14">
         <v>1.3</v>
       </c>
-      <c r="D260" s="14"/>
+      <c r="D260" s="14">
+        <v>1</v>
+      </c>
     </row>
     <row r="261" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A261" s="16"/>
@@ -6118,7 +6120,9 @@
       <c r="C261" s="14">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D261" s="14"/>
+      <c r="D261" s="14">
+        <v>2</v>
+      </c>
     </row>
     <row r="262" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A262" s="16" t="s">
@@ -6130,7 +6134,9 @@
       <c r="C262" s="14">
         <v>0.9</v>
       </c>
-      <c r="D262" s="14"/>
+      <c r="D262" s="14">
+        <v>3</v>
+      </c>
     </row>
     <row r="263" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A263" s="16"/>
@@ -6140,7 +6146,9 @@
       <c r="C263" s="14">
         <v>1</v>
       </c>
-      <c r="D263" s="14"/>
+      <c r="D263" s="14">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="264" spans="1:4" ht="22.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="16"/>
@@ -6208,17 +6216,17 @@
       <c r="C270" s="14"/>
       <c r="D270" s="14"/>
     </row>
-    <row r="271" spans="1:4" s="60" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:4" ht="34" x14ac:dyDescent="0.2">
       <c r="A271" s="31" t="s">
         <v>331</v>
       </c>
       <c r="B271" s="30" t="s">
         <v>403</v>
       </c>
-      <c r="C271" s="59">
-        <v>1.5</v>
-      </c>
-      <c r="D271" s="59">
+      <c r="C271" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="D271" s="14">
         <v>1</v>
       </c>
     </row>

</xml_diff>